<commit_message>
Teams step 1: the host keeps teams in its save and tells every game
Council 2026-10-25 (teams and ownership). Four plain values in the world
save: teams (id -> leader, open, members), team_names, zone_team and
card_owner (plain types only: a mod type inside context_vars would make
every saved value of the mod unreadable if it failed to resolve). Team 0,
the Wanderers, is everyone in no team; an old world has no teams and
nothing changes. The host sends the whole book (TeamsDelta, 980) when a
player joins and when it changes. Internal API Teams.Found/Join/Leave and
console commands emp.team.found/join/leave/list for the bench. Host boxes
"Players can be in teams" and "A base belongs to its team" (Advanced,
off), texts in English, Japanese and Chinese.

Untested in game.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D443"/>
+  <dimension ref="A1:D449"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -7980,6 +7980,108 @@
         </is>
       </c>
     </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_teams</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>チームを組める</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Players can be in teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_teams</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>プレイヤーはチームに入れる。誰がどのチームかはホストのセーブに残る。チームのないプレイヤーは放浪者。オフ：チームはなく、以前どおり</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Players can be in teams, the host keeps who is in which team in its save. A player in no team is a Wanderer. Off: no teams, everything as before</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_team_bases</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>拠点はチームのもの</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>A base belongs to its team</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_team_bases</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>拠点は権利書を読んだプレイヤーのチームのもの。ほかのチームのプレイヤーはそこで箱を開けられず、物を拾えず、建築も拠点の管理もできない。オフ：以前どおり誰でもどの拠点も使える</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>A base belongs to the team of the player who claimed it: the players of another team cannot open its chests, pick up its things, build there or manage it. Off: every player uses every base as before</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>emp_team_belongs</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>これは{0}のものだ。</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>This belongs to {0}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>emp_team_wanderers</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>放浪者</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>the Wanderers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Teams step 8: PvP between teams (host box, off by default)
With "Teams" and the new "PvP between teams" box on, two players of
different real teams are enemies to each other, as two duellists are:
DuelFoePatch now also asks TeamPvp.AreFoes, so a left click, spells and
the bow target the other player in every game (host and guests read the
same shared team book and host rules). Never: Wanderers (team 0), two of
one team, civilized zones (Zone_Civilized: towns, Vernis, guilds...),
the world map, the start zone (stands for the spawn zone of step 6).
A death follows the existing PlayerKill rule (RemotePlayerKillPatch).
No karma (the game gives none for hitting one of the player faction),
no guard call (towns are safe). New rule key 110, config TeamPvp,
settings row team_pvp under Teams, EN/JP/CN texts.

Untested in game.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D449"/>
+  <dimension ref="A1:D451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8082,6 +8082,40 @@
         </is>
       </c>
     </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_team_pvp</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>チーム間のPvP</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>PvP between teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_team_pvp</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>異なるチームのプレイヤーは、町とスポーン地点の外では互いに敵になる。放浪者は誰とも戦わない。プレイヤーが本当に死ぬのは「プレイヤー同士で倒せる」がオンのときだけ。オフ：異なるチームのプレイヤーは戦えない</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Players of different teams are enemies to each other outside towns and the spawn zone. Wanderers fight nobody. A player only really dies if players can kill each other. Off: players of different teams cannot fight</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Teams step 6: spawn zone and a free land deed for a new team
Host choice "Where a new player appears" (with teams): the meadow where a
game starts (default) or the host's map as before; another zone id typed in
the file is used as is. A new player, made or brought, and a returning player
whose team holds no land, travel there once their world is loaded
(TeamSpawnDelta, union 982), the way a player travels alone: needs
independent travel, once per player and hosting, nothing when the host
already stands there.

Host box "A land deed for a new team" (on): the founder receives one deed
("deed", the vanilla claim item): in its bag, or by mail when it is not on
the host's map. Recorded in the save (team_deeds, team -> founder), never
twice for a team nor for a player who founds again after leaving.

Untested in game.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D458"/>
+  <dimension ref="A1:D465"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8235,6 +8235,125 @@
         </is>
       </c>
     </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_team_deed</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>新しいチームに権利書を1枚</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>A land deed for a new team</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_team_deed</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>新しいチームを作ったプレイヤーは土地の権利書を1枚もらう。チームごとに1回、プレイヤーごとに1回。オフ：権利書はゲームどおり商人から買う</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>The player who founds a new team receives one land deed, once per team and once per player. Off: a deed is bought from the merchant as in the game</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_spawn_zone</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>新しいプレイヤーが現れる場所</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Where a new player appears</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_spawn_zone</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>チームがあるとき、新しいプレイヤーと拠点のないチームのプレイヤーは参加するとここへ向かう（一人旅が必要）</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>With teams, a new player and a player whose team has no base go there when they join (needs travelling alone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_spawn_zone_start</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>始まりの草原</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>The meadow where a game starts</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_spawn_zone_host</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>ホストのいるマップ</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>The host's map</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>emp_team_deed_mail</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>{0}のチームの権利書</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>{0}'s team deed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Host box "Public game": anybody who finds the game in the list may join
A game opened by hand was already a public Steam lobby and listed, but the host kicked anyone who was
not a friend, invited, or an account of the world. With the box (off by default) the host lets them in.
A game opened by itself (depot, shared world) is unchanged: only its world's players.
Tested: the switch on the host (OpenToAll false/true), SettingsTableCheck ok. Not tested: a real stranger's
Steam account joining (the bench has one Steam account).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D470"/>
+  <dimension ref="A1:D472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8439,6 +8439,40 @@
         </is>
       </c>
     </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_public_game</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>公開ゲーム</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Public game</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_public_game</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>ゲーム一覧で見つけた人は誰でも参加できる（ホストのSteamフレンドや招待されたプレイヤーだけでなく）。自動で開いたゲーム（保管庫、共有ワールド）はそのワールドのプレイヤーだけ。オフ：フレンドと招待されたプレイヤーのみ</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Anybody who finds the game in the list of games can join, not only the host's Steam friends and invited players. A game opened by itself (depot, shared world) still lets in only its world's players. Off: friends and invited players only</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Host setting: look-only mods are each player's own
Council 2026-10-25 (host mod choice): the game sorts the mods itself, the
host never ticks a content mod out. Server setting LookModsOwn (off by
default): a mod whose every file is a picture, sound or text under
Texture, Texture Replace, Portrait, Sound, Lang or TalkText (no dll, no
table, no map) is left out of the list the host publishes (also from a
depot world's list); the list says so, and a guest that restarts for the
game keeps its own look-only mods on and does not count them as extra.

Test: look_mods_suite 14/14 (sorting, published list on/off, depot list,
session list, extra). Not tested: a real join with a host-only look mod;
a look-only mod that declares a dependency the session switches off.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D472"/>
+  <dimension ref="A1:D474"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8473,6 +8473,40 @@
         </is>
       </c>
     </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_look_mods_own</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>見た目だけのModは各自のもの</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Look-only mods: each player's own</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_look_mods_own</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>見た目だけを変えるMod（画像、肖像、音、翻訳：コード、アイテム、マップなし）は参加者に求められない：そのために再起動する人はおらず、各プレイヤーは自分のものを使い続ける。オフ：参加者はホストのすべてのModが必要</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Mods that only change the look (pictures, portraits, sounds, translations: no code, no items, no maps) are not asked of the players who join: nobody restarts for them, and every player keeps their own. Off: the players who join need every mod of the host</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Team PvP: a player beaten at 0 HP is no longer that team's foe on that map
Council 2026-10-25 (option A, minimal): with player kills off and out of a duel, a strike of a player of another
team that stops a player at 0 hit points ends the fight between them on that map, as a lost duel does. No timer,
no heal, no move. The host decides (TeamPvp.Struck, after RemotePlayerKillPatch's shield), keeps the victim, the
striking team and the victim's map, and tells every game (TeamBeatenDelta, union 978); every game says
"X was beaten by Y." (emp_team_beaten, EN/JP/CN). Cleared with the session (PlayerTrade.WatchSession).
Test: teams2_suite T12 red (4 fails) then 26/26 in Hill Cave; T11's real click of the host already triggered it.
Not covered: a guest reconnecting misses the entries; reviewed (sonnet), its one finding applied.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D474"/>
+  <dimension ref="A1:D475"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8507,6 +8507,23 @@
         </is>
       </c>
     </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>emp_team_beaten</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>{0}は{1}に敗れた。</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>{0} was beaten by {1}.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Settings trim: 7 visible rows, the rest under Advanced, guest told every rule
Council verdict (settings trim): who joins, characters (choose + import),
travel (independent travel + world map clock), combat pace, building,
fights, host leaves stay visible; everything else moves to Advanced, with a
new friends card. Nothing deleted, no default changed, no stored value
rewritten; Classic writes the same.

The guest's rules card also lists an Advanced row that differs from its
default, and six fallbacks the guest was never told now travel with the
session rules (keys 112-117, default true). Texts EN/JA/CN added.

Tests: settings_suite 147/147 (mapping, live, roundtrip, combos, guest,
hidden, fallback, layout), host and guest Player.log without exception.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D475"/>
+  <dimension ref="A1:D486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8524,6 +8524,193 @@
         </is>
       </c>
     </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_characters</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>参加するキャラクター</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Characters of joining friends</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_characters</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>新しいキャラ：毎回新しく作ります。自分のキャラを選ぶ：この世界の自分のキャラを選ぶか、新しく作ります。選ぶか連れてくる：自分のセーブからキャラ（装備、バッグ、お金、名声とカルマ）を連れてくることもできます。</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>New character: a new one each time. Pick one of yours: one of their characters in this world, or a new one. Pick or bring one: also a character from their own saves (gear, bag, gold, fame and karma; the save is never changed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_characters_new</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>新しいキャラ</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>New character</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_characters_pick</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>自分のキャラを選ぶ</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Pick one of yours</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_characters_both</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>選ぶか連れてくる</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Pick or bring one</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_travel</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>旅</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_travel</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>一緒に：全員がホストについていきます。一人で、共有時計：好きな場所へ行けて、ワールドマップで誰かが一歩進むたびに日付が進みます。一人で、自分のペース：同じですが、一人で旅するプレイヤーは世界より先に進み、その時間は本人の満腹度とクエストが払います。</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Together: everyone follows the host. Alone, shared clock: players go anywhere; every step of anyone on the world map moves the date. Alone, own pace: the same, but a player travelling alone runs ahead of the world: its hunger and its own quests pay the hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_travel_together</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>一緒に</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Together</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_travel_alone</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>一人で、共有時計</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Alone, shared clock</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_travel_own_pace</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>一人で、自分のペース</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Alone, own pace</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_sec_friends</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>友人はホストと同じことができる</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Friends can do what the host does</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Join and leave notices read like the game: "Bob joined the game."
The host's message log showed the link's fields ("Player { PeerIndex: 2,
PlayerName:  } connected", and the disconnect reason on a second line).
It now names the player (its Steam name, "A player" while Steam has not
told it) in EN/JP/CN; the link and the reason go to the mod's own log.

Test: reconnect_suite r3 checks the host's log after a deliberate leave
and a rejoin: red before (the raw template), green after; reconnect_suite
72/72, 0 exception. (A text change also needs the game's cached
LangMod/EN/SourceLocalization.json removed: dev/build.ps1 now does it.)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9510" yWindow="2685" windowWidth="31695" windowHeight="18195" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="General" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D486"/>
+  <dimension ref="A1:D487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1173,12 +1173,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>プレイヤー {@Peer} が接続しました</t>
+          <t>{0}がゲームに参加しました。</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Player {@Peer} connected</t>
+          <t>{0} joined the game.</t>
         </is>
       </c>
     </row>
@@ -1190,14 +1190,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>プレイヤー {@Peer} が切断しました
-{DisconnectInfo}</t>
+          <t>{0}がゲームから退出しました。</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Player {@Peer} disconnected
-{DisconnectInfo}</t>
+          <t>{0} left the game.</t>
         </is>
       </c>
     </row>
@@ -8711,6 +8709,23 @@
         </is>
       </c>
     </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>emp_player_someone</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>プレイヤー</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>A player</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Session ping line and client settings read like the game
The ping line used the "P0" percent format, which on this PC's culture
drew an Arabic percent sign the game's font lacks ("Quality: 100 ٪",
seen as "?"): it is now "Ping 0 ms, Quality 100%" ("Ping - (Host)" for
the host). The two Workshop mod toggles of the client settings explained
themselves in "Unticked, ..." paragraphs: one short sentence each now
(EN/JP/CN).

Test: settings_suite texts (new): red before (the Arabic percent sign and
the two paragraphs), green after; settings_suite 165/165, 0 exception.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -884,12 +884,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>遅延: {0}ms{1}</t>
+          <t>遅延 {0} ms{1}</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Ping: {0}ms{1}</t>
+          <t>Ping {0} ms{1}</t>
         </is>
       </c>
     </row>
@@ -901,12 +901,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>遅延: N/A（ホスト）</t>
+          <t>遅延 - （ホスト）</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Ping: N/A (Host)</t>
+          <t>Ping - (Host)</t>
         </is>
       </c>
     </row>
@@ -918,12 +918,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | 品質: {0}</t>
+          <t>, 品質 {0}%</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> | Quality: {0}</t>
+          <t>, Quality {0}%</t>
         </is>
       </c>
     </row>
@@ -4909,12 +4909,12 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>参加するゲームのMODで足りない Workshop のものを、購読せずにダウンロードします。Elin は一度再起動し、自動でゲームに戻ります。MOD一覧は次の起動で元に戻ります。オフ：違うMODを知らせるだけ。</t>
+          <t>参加するゲームに足りない Workshop の MOD を、購読せずにダウンロードします。Elin は一度再起動します。</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Missing Workshop mods of the game you join are downloaded without subscribing. Elin restarts once with those mods and comes back by itself. Your own list returns at the next start. Unticked, you are only told which mods differ.</t>
+          <t>Downloads the Workshop mods you lack for the game you join, without subscribing. Elin restarts once.</t>
         </is>
       </c>
     </row>
@@ -5147,12 +5147,12 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>参加するゲームのMODを Steam アカウントで購読し、自分のMOD一覧に残します。最初の一度だけ再起動し、以降は Elin を閉じても再起動なしで同じゲームに入れます。取り消すには Workshop で購読を解除します。オフ：購読せず取得し、起動後の最初の参加で毎回再起動します。</t>
+          <t>参加するゲームの MOD を Steam で購読し、次からは再起動なしで参加できます。</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Your Steam account subscribes to the mods of the game you join and keeps them on. Elin restarts once, the first time. After that you rejoin the same game with no restart. To undo, unsubscribe on the Workshop. Unticked, Elin restarts at the first join of every start.</t>
+          <t>Subscribes to the game's mods on Steam, so you can rejoin without restarting.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Admin tools S0-S1: a kick that says why and keeps out, bans kept in the world
Council 2026-10-27 (admin tools). A kicked player is told the host's reason
and cannot come back for KickKeepOutMinutes (new setting, 5 by default,
Joining card). Bans by Steam id are kept in the world save (mod_bans), so
they follow the depot, the world copy and a takeover; a banned player is
refused when it connects, before the world is sent, and gets no key in the
Steam lobby. Console: kick <index> [reason], ban <steamid> [reason],
unban <steamid> (also clears a keep-out). The Players tab Kick button uses
the same path.
Tested: admin_suite 14/14 (kick reason shown, kept out, unban, ban
refused, ban kept across save and reload, unban). NOT tested: the lobby
refusal through Steam (needs a second PC).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D493"/>
+  <dimension ref="A1:D503"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8878,6 +8878,182 @@
         </is>
       </c>
     </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>emp_dc_host_kick_why</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>切断: ホストによりキックされました（{0}）</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Disconnected: kicked by the host ({0})</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>emp_dc_banned</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>このワールドから追放されています。</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>You are banned from this world.</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>emp_dc_banned_why</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>このワールドから追放されています：{0}</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>You are banned from this world: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>emp_dc_kick_wait_why</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>このワールドからキックされました。{0}分後にもう一度試してください。</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>You were kicked from this world. Try again in {0} min.</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_kick_keep_out</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>キック後の待ち時間</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Kicked players wait</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_kick_keep_out</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>オフ：キックされたプレイヤーはすぐに戻れる。
+5分：キックされたプレイヤーは5分間戻れない。
+15分：15分間。
+60分：60分間。</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Off: a kicked player can come back at once.
+5 min: a kicked player cannot come back for 5 min.
+15 min: the same for 15 min.
+60 min: the same for 60 min.</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_kick_keep_out_0</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>オフ</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_kick_keep_out_5</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>5分</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_kick_keep_out_15</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>15分</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_kick_keep_out_60</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>60分</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>60 min</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Admin tools S4: mute a player
Mutes by Steam id are kept in the world save (mod_mutes) and told to every
game (ModerationDelta 985, also to players away from the host map). The
host and a player holding a map for others drop a muted player's chat
line, whisper and speech bubble (hard checks, whatever EnforceOwnership
says); the muted player's own game keeps its line and tells it it is
muted. Console and server.cmd: mute|unmute <Steam id> [reason].
Tested: admin_suite 18/18 (muted line not read by the host, the guest is
told, it still reads others, unmute), chat_suite 17/17. NOT tested: a
muted player inside a zone session hosted by another guest, or away.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D503"/>
+  <dimension ref="A1:D504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9054,6 +9054,23 @@
         </is>
       </c>
     </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>emp_ui_muted</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>このワールドでは発言できません（管理者によりミュートされています）。</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>You cannot chat in this world (muted by an admin).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Admin tools S6: members only
New host box MembersOnly (off, Joining card): only the players of the
world come in (a character here, the host's own players, admins, and
accounts let in with allow, kept in mod_members); Steam friends and a
public game's strangers too are refused, at the lobby and when they
connect, told why. Console and server.cmd: allow <Steam id>.
Tested: an unknown account (fake client, identity 30) refused with
emp_dc_members_only, a player of the world comes back, after allow the
same account joins (3/3, logged in admin.log).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D511"/>
+  <dimension ref="A1:D514"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9190,6 +9190,57 @@
         </is>
       </c>
     </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>emp_dc_members_only</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>このワールドには、すでにここでプレイしたプレイヤーだけが参加できます。</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Only the players of this world can join it now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_members_only</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>メンバーのみ</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Members only</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_members_only</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>ここにキャラクターがいるプレイヤー、管理者、許可したプレイヤーだけが参加できる。Steamのフレンドや公開ゲームの知らない人も断られる。オフ：今まで通り。</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Only players with a character here, admins and players let in can join; Steam friends and strangers of a public game are refused. Off: as before.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Permadeath revive: a dead character waits in the character choice
A player who comes back while its character is dead (permadeath with
PermadeathRevive) is asked which character to play: the dead one is
listed as waiting for a revive at a bartender and cannot be picked (the
host refuses it too); it may make or import another meanwhile. Once
revived, even while its player is away, it is played again at the next
join.
Tested: revive_suite 19/19 (new R6: the choice lists 'dead: waiting for
a revive at a bartender', not clickable; R7: the host revives the absent
player, which comes back with that character alive).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D517"/>
+  <dimension ref="A1:D519"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9292,6 +9292,40 @@
         </is>
       </c>
     </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_dead_tag</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>（死亡：バーテンダーでの蘇生待ち）</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>(dead: waiting for a revive at a bartender)</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_dead</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>このキャラクターは死んでいて、バーテンダーでの蘇生を待っています。</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>This character is dead and waits for a revive at a bartender.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Duels can be given up, worn items can be traded; READMEs brought up to date
User 2026-10-27 ('things in the README are outdated, some of what is left
is easy'):
- a duellist gives up through the game's menu on its own character ('Give
  up the duel'): the other wins, as at 0 hit points;
- a worn item may be offered in the trade window; it comes off when the
  trade is made;
- READMEs (EN, FR, ZH, JA): the night choice and idle players, big worlds,
  permadeath revive at the bartender, the dedicated server reachable by
  Steam with hourly backups and its app, the clean host leave, a section
  on public servers (moderation, safety, many players), the new settings,
  limits and what is left as of 27 October (riding fix and world time
  done, give-up and worn items done, issues 5/6 closed).
Tested: duel_suite p1,d10 15/15 (new D10), trade_suite 147/147 (R11 now
expects the worn sword traded and not worn afterwards).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D519"/>
+  <dimension ref="A1:D520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9326,6 +9326,23 @@
         </is>
       </c>
     </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>emp_act_duel_giveup</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>決闘を降参する</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Give up the duel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Report a bug from the game: sent to the developers as a GitHub issue
User 2026-10-27: a button in Client Settings ('Report a bug to the
developers'): the player writes what happened; the mod makes the usual
zip (logs, versions, mods) and sends it with the words to a relay
(dev/relay/worker.js, a Cloudflare Worker holding a key of the ETReport
account): the issue is made on this repository with the player's words
and versions, the logs go to a private repository, the issue's link comes
back to the player. Without an answer from the relay, GitHub's new issue
page opens filled and the zip is shown to drag in.
Tested: the relay answers and refuses posts without the game's header;
the game's send reached it (GitHub then refused the relay's key: 403,
key being fixed); the fallback page opened. The full path with a working
key is not tested yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D520"/>
+  <dimension ref="A1:D526"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9343,6 +9343,110 @@
         </is>
       </c>
     </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>emp_ui_report_send</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>開発者にバグを報告する</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Report a bug to the developers</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>emp_ui_report_send_desc</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>何が起きたかを書くと、ログと一緒に開発者へ送られ、GitHubに公開の報告が作られます。ログ（Steamの名前とIDを含む）は開発者だけが読めます。</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Write what happened: it goes to the developers with your logs, as a public report on GitHub. The logs (they hold Steam names and ids) are only readable by the developers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>emp_ui_report_what</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>何が起きましたか？（何をしていたか、何を期待したか）</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>What happened? (what you were doing, what you expected)</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>emp_ui_report_sending</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>報告を送信中…</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Sending the report…</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>emp_ui_report_page</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>報告ページをブラウザで開きました。デスクトップのzipをドラッグしてSubmitしてください。</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>The report page opened in your browser: drag the zip from your desktop into it and click Submit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>emp_ui_report_sent</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>報告を送信しました：{0}
+ブラウザで開きますか？</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Report sent: {0}
+Open it in your browser?</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Bug reports show the player's Steam name
User 2026-10-27: the public issue made from the game's report button now
says who sent it ("Player (Steam): name"), to ask them more; the text
under the button tells the player that the report shows their Steam name.
Tested: report_check 3/3 (a report sent from the guest game through the
relay made an issue by ETReport showing the guest's Steam name). This
also tests the full in-game path of the report button's sending, which
the previous commit could not.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -9368,12 +9368,12 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>何が起きたかを書くと、ログと一緒に開発者へ送られ、GitHubに公開の報告が作られます。ログ（Steamの名前とIDを含む）は開発者だけが読めます。</t>
+          <t>何が起きたかを書くと、ログと一緒に開発者へ送られ、GitHubに公開の報告が作られます（あなたのSteamの名前が表示されます）。ログ（SteamのIDを含む）は開発者だけが読めます。</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>Write what happened: it goes to the developers with your logs, as a public report on GitHub. The logs (they hold Steam names and ids) are only readable by the developers.</t>
+          <t>Write what happened: it goes to the developers with your logs, as a public report on GitHub that shows your Steam name. The logs (they hold Steam ids) are only readable by the developers.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bug report: a real text box, Enter for a new line, Ctrl+Enter to send
User 2026-10-27: the report's words were typed in the game's one-line
name box (only the end of the text visible). The same input dialog is
now 640x320, its text wrapped and shown from the top with a margin;
Enter starts a new line there (the game closes input dialogs on Enter),
Ctrl+Enter sends, Esc cancels, as the hint above the box says (the game's
input dialog shows no OK button).
Tested: report_box_check 1/1 and its screenshot (five lines, one wrapped,
all shown inside the box, the dialog grown with it). Not tested: the keys
themselves (the bench cannot press Enter or Ctrl+Enter in a minimized
window).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -9385,12 +9385,12 @@
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>何が起きましたか？（何をしていたか、何を期待したか）</t>
+          <t>何が起きましたか？（何をしていたか、何を期待したか）　Enter：改行、Ctrl+Enter：送信、Esc：キャンセル</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
         <is>
-          <t>What happened? (what you were doing, what you expected)</t>
+          <t>What happened? (what you were doing, what you expected)   Enter: new line, Ctrl+Enter: send, Esc: cancel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bug report: the last 30 seconds of the screen go with it
User 2026-10-27 (option 1 of 2): one small picture a second (640 wide,
JPEG 60, made small on the graphics card), the last 30 kept in memory,
written into the report zip as replay/HH-mm-ss.jpg. Client setting
"Send the last 30 seconds of the screen with a bug report" (on by
default); the text under the report button says so. A failure to take a
picture is logged once and the recording stops.
Tested: replay_check 3/3 (after 35 s in game, 30 pictures, 1.4 MB; the
zip with the logs 3.4 MB, under the relay's 6 MB; the newest picture
looked at: right way up, readable). Not measured: the frame time cost.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D544"/>
+  <dimension ref="A1:D545"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9368,12 +9368,12 @@
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>何が起きたかを書くと、ログと一緒に開発者へ送られ、GitHubに公開の報告が作られます（あなたのSteamの名前が表示されます）。ログ（SteamのIDを含む）は開発者だけが読めます。</t>
+          <t>何が起きたかを書くと、ログと最後の30秒の画面と一緒に開発者へ送られ、GitHubに公開の報告が作られます（あなたのSteamの名前が表示されます）。ログと画面（SteamのIDを含む）は開発者だけが見られます。</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>Write what happened: it goes to the developers with your logs, as a public report on GitHub that shows your Steam name. The logs (they hold Steam ids) are only readable by the developers.</t>
+          <t>Write what happened: it goes to the developers with your logs and the last 30 seconds of your screen, as a public report on GitHub that shows your Steam name. The logs and pictures (they hold Steam ids) are only seen by the developers.</t>
         </is>
       </c>
     </row>
@@ -9750,6 +9750,23 @@
       <c r="D544" t="inlineStr">
         <is>
           <t>You have as many characters as this world allows: delete one to make or bring another.</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>emp_ui_cl_record_replay</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>バグ報告に最後の30秒の画面を付ける</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Send the last 30 seconds of the screen with a bug report</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Title screen: Join the official server first, with its player count, or a quiet line when it is not open
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D545"/>
+  <dimension ref="A1:D548"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9770,6 +9770,57 @@
         </is>
       </c>
     </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>emp_ui_official_players</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>現在 {0} 人がプレイ中</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>{0} players online</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>emp_ui_official_closed</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>公式サーバーは今は開いていません</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>The official server is not open right now</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_import_official</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>公式サーバーではキャラクターの持ち込みはできません</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>The official server does not take imported characters</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
World time stage 3: a map a player holds alone stops while that player is away
"Time stops when nobody plays" froze the host's world only. A player alone on
a map of its own (zone lease, no visitor) kept simulating it while away from
the keyboard: with autopause off its clock ran on in real time, and once it
played again its time report pulled the world's date by those hours. Now that
map is frozen and paused too (EmptyWorld.Frozen on the zone authority: its own
player idle and no visitor connected). A catch-up with the world still comes.
Same host setting, its description says so (EN/JP/CN).

Test: bench/world_time_stage3.py (ALONE: frozen, an hour of waiting and 15 s do
not move the guest's date, the host's 2 h still reach it, active again the hour
passes and the world moves by that hour only, box off as before; WORLD: hunt5
W08). Not run on the game in this commit (worker without the bench).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -8869,12 +8869,12 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>接続中で操作しているプレイヤーがいない間、世界の日付は止まります。ホストも離席中なら数えません。オフ：従来どおり時間が進みます。</t>
+          <t>接続中で操作しているプレイヤーがいない間、世界の日付は止まります。ホストも離席中なら数えません。一人で自分のマップにいるプレイヤーが離席している間は、そのマップの時間も止まります。オフ：従来どおり時間が進みます。</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>With no player connected and active (the host counts unless away), the date of the world stands still. Off: time goes on as before.</t>
+          <t>With no player connected and active (the host counts unless away), the date of the world stands still; so does the map of a player alone there and away. Off: time goes on as before.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
World time stage 4: "Quests wait for absent players" as a host setting
A returning player's personal quest deadlines already moved by the time the
world went on without it (PlayerLastSeen, ResumeAfterAbsence, since 0.26.1082),
with no box for the host. Now a host setting in World rules > time details
(AbsentQuestsWait, on: the shipped behaviour; shown under personal quests).
Off: the quests run out with the world as before; the date the player came
back is still kept, so turning it on later counts only the next absence.
Texts EN/JP/CN.

Test: bench/world_time_stage4.py (ON: the absent guest's quest keeps its time
and its hunger, a second guest present all along lives the 3 days; OFF: the
quest comes back 3 days shorter). Not run on the game in this commit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D545"/>
+  <dimension ref="A1:D547"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9770,6 +9770,40 @@
         </is>
       </c>
     </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_absent_quests_wait</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>不在の間はクエストが待つ</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Quests wait for absent players</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_absent_quests_wait</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>ゲームを離れたプレイヤーのクエストは残り時間を保ちます。戻ったとき、留守中に世界で過ぎた日数が期限に加わります。オフ：世界の時間とともに期限が過ぎます。</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>A player who left the game finds its quests with the time they had left: the days the world went on without it are added to their deadlines. Off: they run out as the world goes on.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Teams learn on their own (1/7): ledger, seeding, save-time union
Host option "Teams learn on their own" (TeamKnowledge, off, under Teams; rule key 1010). The host's save keeps
what each team knows (recipes learnt, recipes crafted once, codex) in team_lore, with a schema version. Ticking
the box gives every team, the Wanderers too, a copy of what the world knows (once); unticking it gives the world
back everything any team learnt and empties the ledger. While the game saves, the Player object holds the union
of every team, so a save opened without the mod or with the box off keeps everything. Console: team.lore.

Not tested in game yet (bench script in a later commit).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D545"/>
+  <dimension ref="A1:D547"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9770,6 +9770,40 @@
         </is>
       </c>
     </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_team_knowledge</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>チームごとに学ぶ</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Teams learn on their own</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_team_knowledge</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>各チームが自分のレシピ、作ったものの記録、図鑑を持ちます。プレイヤーが覚えたことはチームの仲間も覚え、ほかのチームは覚えません。物語の報酬のレシピは全チームに届き、セーブには全チームの知識が残ります。オフ：全員で一つのレシピと図鑑を共有します（これまで通り）。</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Each team has its own recipes, list of things crafted and codex: what a player learns, its teammates learn too, the other teams do not. Recipes the story gives reach every team, and the save keeps what every team knows. Off: one book of recipes and one codex for everyone, as before.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Setting: each player has their own journal (OwnJournal, rules key 150, on by default)
A fallback box like the other "every player gets their own" ones: on, a
player's journal tells about that player; off, a guest's journal shows the
host's after a trip, as before. An older host sends no key 150: off.
On by default, it only makes guests equal to the host. Texts EN/JP/CN.
Test: bench/journal_check.py j0 (written, not run: no game here).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D545"/>
+  <dimension ref="A1:D547"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9770,6 +9770,40 @@
         </is>
       </c>
     </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_own_journal</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>日誌はプレイヤーごと</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Each player has their own journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_own_journal</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>メッセージの履歴と自分の記録（採掘・死亡・睡眠の回数）は旅をしても自分のものです。図鑑・討伐数・世界の日付は共通です。オフ：旅のあとはホストの日誌が見えます。</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Each player keeps its own message history and its own records (digging, deaths, nights slept) from trip to trip; the codex, kills and the world's dates stay shared. Off: after a trip, a player's journal shows the host's.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Character export 4/5: texts (EN, JP, CN)
The setting (emp_ui_sv_cfg/desc_export_chara) and the choice screen, notices and solo-load messages.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D576"/>
+  <dimension ref="A1:D592"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -10303,6 +10303,278 @@
         </is>
       </c>
     </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_export_chara</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>キャラをソロのセーブへ連れて行ける</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Friends can take a character to a solo save</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_export_chara</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>キャラの一覧から、自分のソロのセーブへキャラを連れて行きます。そのセーブを次に読み込むと、そのセーブのキャラと入れ替わります（先にセーブのコピーを作ります）。キャラはこの世界を離れ、セーブからの持ち込みで戻るか、そのまま呼び戻すまで遊べません。持ち込みがオンのときだけ。オフ：連れて行けません。</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>From the character list, friends take a character to one of their solo saves, where it replaces that save's character when it is next loaded (a copy of the save is made first). It leaves this world until it comes back by being brought from that save, or is brought back unchanged. Only with saved characters allowed. Off: they cannot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_export</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>キャラをソロのセーブへ連れて行く…</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Take a character to a solo save…</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_export_pick</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>どのキャラをソロのセーブへ連れて行きますか？</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>Which character goes to a solo save?</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_export_save</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>どのセーブへ？そのセーブのキャラは入れ替わります。</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>Into which save? Its own character will be replaced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_export_confirm</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>#1 はこの世界を離れ、#2 へ行きます。先にそのセーブのコピーを作ります。次にそのセーブを読み込むと、#1 がそのセーブのキャラと入れ替わり、元のキャラはコピーにだけ残ります。#1 は、そのセーブからの持ち込みで戻るまで、ここでは遊べません。よろしいですか？</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>#1 leaves this world for #2. A copy of that save is made first. When you next load it, #1 takes the place of its character, which then stays only in the copy. #1 cannot be played here until it is brought back from that save. Go?</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_exported</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>キャラはソロのセーブで待っています。タイトル画面からそのセーブを読み込んでください。</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>The character waits in your solo save: load that save from the title screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_export_fail</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>キャラをそのセーブへ連れて行けませんでした。この世界に残ります。</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>The character could not be taken to that save. It stays in this world.</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_export_stale</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>このキャラの旅は終わっています（呼び戻し済み、またはすでに戻っています）。もう一度は来られません。</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>This character's trip is over (brought back, or already returned): it cannot come in again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_away_tag</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>（ソロのセーブ中：#1）</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>(in a solo save: #1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_away</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>このキャラはソロのセーブにいます。</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>This character is in a solo save.</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_recall</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>そのまま呼び戻す…</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>Bring back unchanged…</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_recall_confirm</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>#1 を出発したときのまま呼び戻しますか？ソロのセーブにいるキャラは、もうここへは戻れません。</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>Bring #1 back as it left? The one in the solo save can then never come here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_recalled</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>キャラを出発したときのまま呼び戻しました。</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>The character is back as it left.</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_export_arrived</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>#1 が協力プレイの世界から来て、このセーブのキャラと入れ替わりました（前のセーブはバックアップにあります）。</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>#1 came from a co-op world and took the place of this save's character (the save as it was is in the backups).</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>emp_ui_chara_export_load_fail</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>協力プレイの世界から来たキャラを、このセーブへ入れられませんでした。セーブはそのままです。キャラは ElinMP/Incoming で待っています。</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>A character from a co-op world could not be brought into this save. The save is as it was; the character waits in ElinMP/Incoming.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Team story 1/5: a ledger of each team's story, seeded from the world's, the save keeps the world team's
Host option "Teams live their own story" (experimental, off, needs Teams; council
2026-10-28). The story is the main quest and the exploration of Nymelle with the
dialog choices told to Ash and Fiama (ash1, tutorial1, fiama1). Ticking the box gives
every team the story point the world is at and pins the world team (the host's team);
Game.Save writes the world team's story in the quest log, so a save opened without the
mod or with the box off goes on with it. Unticked: the world team's story stays, the
ledger is emptied. A newer ledger schema turns every swap off. Console: emp.team.story,
emp.team.story_world <team> (the host's explicit choice of the world team).

Not tested in game yet (bench scripts come with commit 5).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D610"/>
+  <dimension ref="A1:D616"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -10881,6 +10881,108 @@
         </is>
       </c>
     </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_team_own_story</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>チームごとの物語（実験的）</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Teams live their own story (experimental)</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_team_own_story</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>実験的。各チームが自分のメインストーリーを進める：アッシュのクエストとニメルの探索、物語の会話はチームごと。チェックした時点の物語の進み具合から全チームが始める。ファリスは最初のチームの拠点にだけ加わる。他のチームがすでに攻略した階に着いたチームは、そこから物語を進める。ワールドチーム（チェックした時のホストのチーム）の物語がセーブに残る：チェックを外す、またはMODなしでセーブを開くと、そのチームの物語で続く。チームが必要。</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>Experimental. Each team lives its own main story: Ash's quest and the exploration of Nymelle, and their dialogs, are its own. Every team starts at the story point the world is at when the box is ticked. Farris joins the base of the first team only; a team reaching a floor another team already cleared takes the story on from there. The save keeps the story of the world team (the host's team when the box is ticked): unticked, or the save opened without the mod, the world goes on with that team's story. Needs Teams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>emp_team_story_moved</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>日誌は今のチームの物語に従う。</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Your journal now follows your team's story.</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>emp_team_story_caught_up_farris</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>ファリスは他のチームとすでにここを去った。あなたのチームはそこから物語を進める。</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Farris already left here with another team: your team takes the story on from there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>emp_team_story_caught_up_boss</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>ニメルの守護者は他のチームがすでに倒した。あなたのチームはそこから物語を進める。</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Another team already defeated the guardian of Nymelle: your team takes the story on from there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>emp_team_story_caught_up_crystal</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>水晶のそばのフィアマの話は他のチームがすでに聞いた。あなたのチームはそこから物語を進める。</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Another team already heard Fiama by the crystal: your team takes the story on from there.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Team knowledge on the same owners as the story: a team shares one book, a player without a team has its own
User, 2026-10-28: separating by player and team means the codex and the recipes too.
TeamKnowledge now keys its ledger by StoryOwner (team id, or -chara uid for a player
without a team; the old Wanderers entry is only read as a fallback for a ledger of the
time of teams), with the same move rule (join: the team's book, or the joiner's when the
team has none; leave: a copy of the team's as the player's own; a gone team keeps its
entry so the save's union keeps what it knew). The box no longer needs Teams, stays off
by default and reads on while hosting the official public server (row greyed with the
reason). The vanilla save still gets the union of every book.

Not tested in game yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -9954,12 +9954,12 @@
       </c>
       <c r="C556" t="inlineStr">
         <is>
-          <t>チームごとに学ぶ</t>
+          <t>プレイヤーとチームごとに学ぶ</t>
         </is>
       </c>
       <c r="D556" t="inlineStr">
         <is>
-          <t>Teams learn on their own</t>
+          <t>Each player or team learns on its own</t>
         </is>
       </c>
     </row>
@@ -9971,12 +9971,12 @@
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>各チームが自分のレシピ、作ったものの記録、図鑑を持ちます。プレイヤーが覚えたことはチームの仲間も覚え、ほかのチームは覚えません。物語の報酬のレシピは全チームに届き、セーブには全チームの知識が残ります。オフ：全員で一つのレシピと図鑑を共有します（これまで通り）。</t>
+          <t>各プレイヤーが自分のレシピ、作ったものの記録、図鑑を持つ。チームの仲間は一つを共有し、チームのないプレイヤーは自分だけのものを持つ。物語の報酬のレシピは全員に配られ、セーブには全員の知識が残る。オフ：全員が一つのレシピと図鑑を共有する（従来どおり）。</t>
         </is>
       </c>
       <c r="D557" t="inlineStr">
         <is>
-          <t>Each team has its own recipes, list of things crafted and codex: what a player learns, its teammates learn too, the other teams do not. Recipes the story gives reach every team, and the save keeps what every team knows. Off: one book of recipes and one codex for everyone, as before.</t>
+          <t>Each player has its own recipes, crafted list and codex; teammates share one, a player without a team has its own. Recipes given by the story reach everyone, and the save keeps everything anyone learnt. Off: everyone shares one book of recipes and one codex, as before.</t>
         </is>
       </c>
     </row>
@@ -10991,12 +10991,12 @@
       </c>
       <c r="C617" t="inlineStr">
         <is>
-          <t>公式サーバーでは常にオン：プレイヤーとチームごとの物語。</t>
+          <t>公式サーバーでは常にオン：プレイヤーとチームごと。</t>
         </is>
       </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>Always on for the official public server: a story for each player and team.</t>
+          <t>Always on for the official public server: one for each player and team.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
World time stage 6 step 1: the Living world rule, a host choice (off by default)
LivingWorldMinutes (EmpConfig.Server, NetSessionRules key 175): real minutes per game day, 0 off.
Settings row "Living world (real-time clock)" in Time details: Off / 20 / 40 / 60 / 120 min,
texts in EN, JP and CN. Nothing reads it yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D617"/>
+  <dimension ref="A1:D624"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11000,6 +11000,133 @@
         </is>
       </c>
     </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_living_world</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>生きている世界（現実の時間）</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>Living world (real-time clock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_living_world</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>オフ：従来どおり、日付はプレイヤーのターンとともに進みます。
+20分：世界の時計が現実の時間に従い、現実の20分で1日が過ぎます。プレイヤーが動いていても立ち止まっていても同じです。誰も遊んでいない間は止まり（「誰も遊んでいない間は時間が止まる」）、夜のルールが許す睡眠は朝まで続きます。各プレイヤーの行動は今までどおり自分のターンで進みます。
+40分：同じく、現実の40分で1日。
+60分：同じく、現実の1時間で1日。
+120分：同じく、現実の2時間で1日。</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Off: the date moves with the players' turns, as before.
+20 min: the clock of the world follows real time, a day every 20 real minutes, whether the players act or stand still. It stops while nobody plays ("Time stops when nobody plays"), and a night slept as the night rule allows runs to the morning. Each player's own acts still go by its own turns.
+40 min: the same, a day every 40 real minutes.
+60 min: the same, a day every real hour.
+120 min: the same, a day every 2 real hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_living_world_0</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>オフ</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_living_world_20</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>1日 = 20分</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>A day = 20 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_living_world_40</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>1日 = 40分</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>A day = 40 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_living_world_60</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>1日 = 1時間</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>A day = 1 hour</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_living_world_120</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>1日 = 2時間</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>A day = 2 hours</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Texts: 42 Japanese and Chinese fixes to the game's own terms
Reviewed 269 rows added since 2026-10-26 against the game's CN/JP sources:
oren (not gold) for money, Nymelle, Farris, Fiama's magic stone, deeds,
karma (善恶值), arena (斗技场), moongate, sky helm, sky ticket, landing portal,
Loytel, Big Daddy, the exotic merchant, the hearth stone, tax bill; 房主 for
the host in recent CN rows. English unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -3838,7 +3838,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>友人は拠点を変更できません（研究、炉の技能、方針、名前、設定、住人、建築）。オフ：全員ができます。拠点を完全に手放せるのはホストだけです。</t>
+          <t>友人は拠点を変更できません（研究、盟約の石の技能、方針、名前、設定、住人、建築）。オフ：全員ができます。拠点を完全に手放せるのはホストだけです。</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>店の仕入れはマップ上で最も良いプレイヤーの特性で決まり、特別な棚（結婚とカセットの店、ロイテルのマート、異国の商人）は店を開いたプレイヤーの進行に従います。オフ：ホストの進行（元のゲームと同じ）。</t>
+          <t>店の仕入れはマップ上で最も良いプレイヤーの特性で決まり、特別な棚（結婚とカセットの店、ロイテルのマート、舶来品商人）は店を開いたプレイヤーの進行に従います。オフ：ホストの進行（元のゲームと同じ）。</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
@@ -7727,7 +7727,7 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>友人は着陸ポータルで一人で移動する</t>
+          <t>友人は地上転移ポータルで一人で移動する</t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>友人の着陸ポータルは、その友人だけをゲートのある場所へ運びます。ホストは動きません。</t>
+          <t>友人の地上転移ポータルは、その友人だけをゲートのある場所へ運びます。ホストは動きません。</t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>友人も空の舵を使える</t>
+          <t>友人も飛空艇の舵を使える</t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
@@ -7778,7 +7778,7 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>友人の空の舵は、ホストの行き先の一覧をその友人の画面に出し、その友人の空の切符で払います。ゲートの場所は全員で変わります。</t>
+          <t>友人の飛空艇の舵は、ホストの行き先の一覧をその友人の画面に出し、その友人の旅空券で払います。ゲートの場所は全員で変わります。</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
@@ -10124,7 +10124,7 @@
       </c>
       <c r="C566" t="inlineStr">
         <is>
-          <t>決闘を申し込む側が金貨の賭け金（なし、100、1,000、または二人のうち少ない方の所持金すべて）を決め、相手は答えるときにそれを見ます。両者が賭け金を出し、勝者が全部受け取ります。勝者なしで終わったとき（離れた、接続が切れた、ゲームが止まった）は各自に返されます。降参すると失います。</t>
+          <t>決闘を申し込む側がオレンの賭け金（なし、100、1,000、または二人のうち少ない方の所持金すべて）を決め、相手は答えるときにそれを見ます。両者が賭け金を出し、勝者が全部受け取ります。勝者なしで終わったとき（離れた、接続が切れた、ゲームが止まった）は各自に返されます。降参すると失います。</t>
         </is>
       </c>
       <c r="D566" t="inlineStr">
@@ -10175,7 +10175,7 @@
       </c>
       <c r="C569" t="inlineStr">
         <is>
-          <t>金貨 {0} 枚</t>
+          <t>{0}オレン</t>
         </is>
       </c>
       <c r="D569" t="inlineStr">
@@ -10209,7 +10209,7 @@
       </c>
       <c r="C571" t="inlineStr">
         <is>
-          <t>{0}が金貨 {1} 枚ずつを賭けて決闘を申し込んできた。誰も死なないが、使った物は戻らない。受けますか？</t>
+          <t>{0}が{1}オレンずつを賭けて決闘を申し込んできた。誰も死なないが、使った物は戻らない。受けますか？</t>
         </is>
       </c>
       <c r="D571" t="inlineStr">
@@ -10226,7 +10226,7 @@
       </c>
       <c r="C572" t="inlineStr">
         <is>
-          <t>{0} に金貨 {1} 枚ずつを賭けて決闘を申し込みました…</t>
+          <t>{0} に{1}オレンずつを賭けて決闘を申し込みました…</t>
         </is>
       </c>
       <c r="D572" t="inlineStr">
@@ -10243,7 +10243,7 @@
       </c>
       <c r="C573" t="inlineStr">
         <is>
-          <t>賭け金として金貨 {0} 枚を出した。</t>
+          <t>賭け金として{0}オレンを出した。</t>
         </is>
       </c>
       <c r="D573" t="inlineStr">
@@ -10260,7 +10260,7 @@
       </c>
       <c r="C574" t="inlineStr">
         <is>
-          <t>賭け金の金貨 {0} 枚を手に入れた！</t>
+          <t>賭け金の{0}オレンを手に入れた！</t>
         </is>
       </c>
       <c r="D574" t="inlineStr">
@@ -10362,7 +10362,7 @@
       </c>
       <c r="C580" t="inlineStr">
         <is>
-          <t>土地を持つチームごとに毎月の税の請求書が届きます。自分の土地の分だけで、メンバーの最も高い名声で計算されます（どのチームのものでもない土地は放浪者の分）。未払いの請求書はチームごとに数え、4枚以上になるとそのチームのプレイヤーだけがカルマを失います。オフ：世界全体で請求書は一枚（これまで通り）。</t>
+          <t>土地を持つチームごとに毎月の税金請求書が届きます。自分の土地の分だけで、メンバーの最も高い名声で計算されます（どのチームのものでもない土地は放浪者の分）。未払いの請求書はチームごとに数え、4枚以上になるとそのチームのプレイヤーだけがカルマを失います。オフ：世界全体で請求書は一枚（これまで通り）。</t>
         </is>
       </c>
       <c r="D580" t="inlineStr">
@@ -10379,7 +10379,7 @@
       </c>
       <c r="C581" t="inlineStr">
         <is>
-          <t>{0}の税の請求書：{1}</t>
+          <t>{0}の税金請求書：{1}</t>
         </is>
       </c>
       <c r="D581" t="inlineStr">
@@ -10413,7 +10413,7 @@
       </c>
       <c r="C583" t="inlineStr">
         <is>
-          <t>未払いの税の請求書：{0}</t>
+          <t>未払いの税金請求書：{0}</t>
         </is>
       </c>
       <c r="D583" t="inlineStr">
@@ -10583,7 +10583,7 @@
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>ナイメルの後</t>
+          <t>ナイミールの後</t>
         </is>
       </c>
       <c r="D593" t="inlineStr">
@@ -10906,7 +10906,7 @@
       </c>
       <c r="C612" t="inlineStr">
         <is>
-          <t>実験的。各プレイヤーが自分のペースでメインストーリーを進める（アッシュのクエスト、ニメルの探索とその会話）。チームの仲間は一緒：チームは一つの物語を共有し、チームのないプレイヤーは自分だけの物語を持つ。チェックした時点の物語の進み具合から全員が始める。ファリスは最初の拠点にだけ加わる。他の人がすでに攻略した階に着いたプレイヤーやチームは、そこから物語を進める。セーブにはホスト自身の物語が残る：チェックを外す、またはMODなしでセーブを開くと、その物語で続く。オフ：全員が一つの物語の進み具合を共有する（従来どおり）。</t>
+          <t>実験的。各プレイヤーが自分のペースでメインストーリーを進める（アッシュのクエスト、ナイミールの探索とその会話）。チームの仲間は一緒：チームは一つの物語を共有し、チームのないプレイヤーは自分だけの物語を持つ。チェックした時点の物語の進み具合から全員が始める。ファリスは最初の拠点にだけ加わる。他の人がすでに攻略した階に着いたプレイヤーやチームは、そこから物語を進める。セーブにはホスト自身の物語が残る：チェックを外す、またはMODなしでセーブを開くと、その物語で続く。オフ：全員が一つの物語の進み具合を共有する（従来どおり）。</t>
         </is>
       </c>
       <c r="D612" t="inlineStr">
@@ -10957,7 +10957,7 @@
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>ニメルの守護者は他の人がすでに倒した。あなたの物語はそこから進む。</t>
+          <t>ナイミールの守護者は他の人がすでに倒した。あなたの物語はそこから進む。</t>
         </is>
       </c>
       <c r="D615" t="inlineStr">
@@ -10974,7 +10974,7 @@
       </c>
       <c r="C616" t="inlineStr">
         <is>
-          <t>水晶のそばのフィアマの話は他の人がすでに聞いた。あなたの物語はそこから進む。</t>
+          <t>魔石のそばのフィアマの話は他の人がすでに聞いた。あなたの物語はそこから進む。</t>
         </is>
       </c>
       <c r="D616" t="inlineStr">

</xml_diff>

<commit_message>
Dedicated server rests while nobody is connected
ServerRestsWhenEmpty (host setting, off): a -empserver game with no peer runs at 5 frames
a second with its sound paused, and gets its own frame rate back from the next frame a
peer connects. The world is already frozen while empty (EmptyWorld), so nothing of the
simulation is lost; this only stops the always-on machine from burning a core for an
empty world. Not tested in game yet (bench/server_rest_check.py, not run).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D625"/>
+  <dimension ref="A1:D627"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11144,6 +11144,40 @@
         </is>
       </c>
     </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_server_rests</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>無人のとき専用サーバーを休ませる</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Dedicated server rests when empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_server_rests</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>専用サーバー（-empserver）に誰も接続していない間、毎秒5フレームで動き、音を止めます。誰かが接続するとすぐに元の速さに戻ります。オフ：常にゲームの通常のフレームレートで動きます。</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>While nobody is connected, a dedicated server (-empserver) runs at 5 frames a second with its sound stopped, and goes back to full speed as soon as a player connects. Off: it always runs at the game's own frame rate.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Texts: English says orens, the game's currency name, instead of gold
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -2390,7 +2390,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Gold: {0}</t>
+          <t>Orens: {0}</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>How much gold?</t>
+          <t>How many orens?</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Click another player to trade items and gold; both must confirm.</t>
+          <t>Click another player to trade items and orens; both must confirm.</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2849,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Friends bring the character, gear, bag, gold, fame and karma from their own saves, never changing them; not companions, base, quests or bank. Off: they cannot.</t>
+          <t>Friends bring the character, gear, bag, orens, fame and karma from their own saves, never changing them; not companions, base, quests or bank. Off: they cannot.</t>
         </is>
       </c>
     </row>
@@ -3648,7 +3648,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Friends use build mode in the base (floors, walls, furniture, mining, cutting) and pay the gold and materials. Off: only the host builds.</t>
+          <t>Friends use build mode in the base (floors, walls, furniture, mining, cutting) and pay the orens and materials. Off: only the host builds.</t>
         </is>
       </c>
     </row>
@@ -5577,7 +5577,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Orens</t>
         </is>
       </c>
     </row>
@@ -5645,7 +5645,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>{0} now offers {1} gold.</t>
+          <t>{0} now offers {1} orens.</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>{0}: {1} gold, {2}</t>
+          <t>{0}: {1} orens, {2}</t>
         </is>
       </c>
     </row>
@@ -6549,7 +6549,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>Everyone builds and manages: all players use build mode in the base and manage it (research, policies, names, residents); friends pay their own gold and materials.
+          <t>Everyone builds and manages: all players use build mode in the base and manage it (research, policies, names, residents); friends pay their own orens and materials.
 Everyone manages, only the host builds: all players manage the base; only the host uses build mode.
 Only the host: only the host builds and manages the base.</t>
         </is>
@@ -8418,7 +8418,7 @@
         <is>
           <t>New character: friends make a new character each time they join.
 Pick one of yours: friends pick one of their characters in this world, or make a new one.
-Pick or bring one: friends can also bring a character from their own saves (gear, bag, gold, fame, karma); the save is never changed.</t>
+Pick or bring one: friends can also bring a character from their own saves (gear, bag, orens, fame, karma); the save is never changed.</t>
         </is>
       </c>
     </row>
@@ -10129,7 +10129,7 @@
       </c>
       <c r="D566" t="inlineStr">
         <is>
-          <t>The challenger of a duel names a stake in gold (none, 100, 1,000 or all the poorer of the two has), shown in the box the other one answers; both put it down and the winner takes both. When the duel ends without a winner (a player leaves or drops out, the game stops) each one gets its stake back; giving up loses it.</t>
+          <t>The challenger of a duel names a stake in orens (none, 100, 1,000 or all the poorer of the two has), shown in the box the other one answers; both put it down and the winner takes both. When the duel ends without a winner (a player leaves or drops out, the game stops) each one gets its stake back; giving up loses it.</t>
         </is>
       </c>
     </row>
@@ -10180,7 +10180,7 @@
       </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>{0} gold</t>
+          <t>{0} orens</t>
         </is>
       </c>
     </row>
@@ -10214,7 +10214,7 @@
       </c>
       <c r="D571" t="inlineStr">
         <is>
-          <t>{0} challenges you to a duel for a stake of {1} gold each. Nobody dies, but what you use up stays used. Accept?</t>
+          <t>{0} challenges you to a duel for a stake of {1} orens each. Nobody dies, but what you use up stays used. Accept?</t>
         </is>
       </c>
     </row>
@@ -10231,7 +10231,7 @@
       </c>
       <c r="D572" t="inlineStr">
         <is>
-          <t>You challenge {0} to a duel for {1} gold each…</t>
+          <t>You challenge {0} to a duel for {1} orens each…</t>
         </is>
       </c>
     </row>
@@ -10248,7 +10248,7 @@
       </c>
       <c r="D573" t="inlineStr">
         <is>
-          <t>You put down a stake of {0} gold.</t>
+          <t>You put down a stake of {0} orens.</t>
         </is>
       </c>
     </row>
@@ -10265,7 +10265,7 @@
       </c>
       <c r="D574" t="inlineStr">
         <is>
-          <t>You take the stakes: {0} gold!</t>
+          <t>You take the stakes: {0} orens!</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Affinity per player: host setting (off by default), rules key 135, texts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D625"/>
+  <dimension ref="A1:D627"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11144,6 +11144,40 @@
         </is>
       </c>
     </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_affinity_per_player</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>好感度はプレイヤーごと</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Affinity per player</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_affinity_per_player</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>住人は各プレイヤーに別々の好感度を持つ。贈り物・会話・依頼は行ったプレイヤーにだけ数えられ、会話の選択肢は話しているプレイヤーの好感度に従う。オフ：住人ごとに一団で一つの好感度（従来通り）。</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>Each resident has its own affinity with each player: gifts, talks and quests count for the player who made them, and the talk options (invite, marry, sleep beside) follow the one who talks. Off: one affinity per resident for the whole group, as before.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Own story: every dialog flag and Fiama's story flags are the story owner's
With 'Each player or team lives its own story' on, the story bundle holds
every Player.dialogFlags entry (what any drama remembers was said or chosen:
the user's 'etc.' is the story-owner's progress), not only Ash's and Fiama's
(StoryBundle.AllDialog, key 10), and Fiama's own story flags (storyFiama and
her dreams). Every 'd:' flag is routed to the owner's players and applied on
the host inside the sender's story. An older ledger keeps its Ash/Fiama
choices over the world's other dialogs, once at load. The save and the box
off keep the world owner's, as before. The setting's text names what the
story now holds.

Bench: bench/team_story_dialogs.py (2 windows), not run here.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -10906,12 +10906,12 @@
       </c>
       <c r="C612" t="inlineStr">
         <is>
-          <t>実験的。各プレイヤーが自分のペースでメインストーリーを進める（アッシュのクエスト、ニメルの探索とその会話）。チームの仲間は一緒：チームは一つの物語を共有し、チームのないプレイヤーは自分だけの物語を持つ。チェックした時点の物語の進み具合から全員が始める。ファリスは最初の拠点にだけ加わる。他の人がすでに攻略した階に着いたプレイヤーやチームは、そこから物語を進める。セーブにはホスト自身の物語が残る：チェックを外す、またはMODなしでセーブを開くと、その物語で続く。オフ：全員が一つの物語の進み具合を共有する（従来どおり）。</t>
+          <t>実験的。各プレイヤーが自分のペースで物語を進める（アッシュのクエスト、ニメルの探索、すべての会話の選択、キーアイテム、ロイテルへの借金と追加の税）。チームの仲間は一緒：チームは一つの物語を共有し、チームのないプレイヤーは自分だけの物語を持つ。チェックした時点の物語の進み具合から全員が始める。ファリスは最初の拠点にだけ加わる。他の人がすでに攻略した階に着いたプレイヤーやチームは、そこから物語を進める。セーブにはホスト自身の物語が残る：チェックを外す、またはMODなしでセーブを開くと、その物語で続く（キーアイテムは誰かが得た分すべて）。オフ：全員が一つの物語の進み具合を共有する（従来どおり）。</t>
         </is>
       </c>
       <c r="D612" t="inlineStr">
         <is>
-          <t>Experimental. Each player lives the main story at its own pace (Ash's quest, the exploration of Nymelle and their dialogs), teammates together: a team shares one story, a player without a team has its own. Everyone starts at the story point the world is at when the box is ticked. Farris joins the first base only; a player or team reaching a floor someone already cleared takes the story on from there. The save keeps the host's own story: unticked, or the save opened without the mod, the world goes on with it. Off: all players share one story progression, as before.</t>
+          <t>Experimental. Each player lives the story at its own pace (Ash's quest, the exploration of Nymelle, every dialog choice, the key items, Loytel's debt and the extra tax), teammates together: a team shares one story, a player without a team has its own. Everyone starts at the story point the world is at when the box is ticked. Farris joins the first base only; a player or team reaching a floor someone already cleared takes the story on from there. The save keeps the host's own story: unticked, or the save opened without the mod, the world goes on with it (the key items: all that anyone got). Off: all players share one story progression, as before.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Teams: host setting 'Teams keep their own bank and delivery box' and its ledger
The box needs Teams, is off by default and is forced on for the official server. The ledger (owner -> bank and
delivery box) is a host save property with a schema number, like the teams' knowledge. Rules key 133.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D632"/>
+  <dimension ref="A1:D634"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11263,6 +11263,40 @@
         </is>
       </c>
     </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_team_boxes</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>チームごとの銀行と配達ボックス</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Teams keep their own bank and delivery box</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_team_boxes</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>各チーム（チームのいないプレイヤーは単独）が自分の銀行と配達ボックスを持ちます。古い箱の中身は全員で共有のままです。チームが有効な場合のみ。オフにすると、各チームの箱は共有の箱に戻されます。</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Each team (a player without a team: alone) has its own bank and delivery box. What the old shared boxes hold stays shared, and everyone can still take from them. Needs Teams. Unticked, every team's box is merged back into the shared one.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Parcels per team: tag, label, delivery by unit, mail box owner
A parcel sent for a player carries its character uid and shows its name. With the teams' boxes on, a
tagged parcel is delivered only into a base of the recipient's unit (its owned mail box, else an ownerless
one, else the unit's delivery box, which is also where a unit without a base gets it). A mail box is owned
by its installer and the owner changes it from the item's menu (CardSettingDelta.MailOwner).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D634"/>
+  <dimension ref="A1:D637"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11297,6 +11297,57 @@
         </is>
       </c>
     </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>emp_parcel_for</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>{0}宛て</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>for {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>emp_mailbox_owner</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>郵便受けの持ち主: {0}</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Mailbox owner: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>emp_mailbox_everyone</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>みんな</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>everyone</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Team tab: the teams get a page in the Elin Together menu (found with a typed name, join, leave, accept, refuse, members, lands)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D634"/>
+  <dimension ref="A1:D650"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11297,6 +11297,278 @@
         </is>
       </c>
     </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>emp_ui_tab_team</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>チーム</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>emp_tab_team</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>チーム</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>emp_ui_team_title</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>チーム</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>emp_ui_team_none</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>あなたはチームに入っていません（放浪者です）。</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>You are not in a team (you are a Wanderer).</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>emp_ui_team_name_ask</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>新しいチームの名前</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Name of the new team</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>emp_ui_team_mine</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>あなたのチーム：{0}</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Your team: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>emp_ui_team_leader</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>リーダー：{0}（{1}）</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Leader: {0} ({1})</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>emp_ui_team_open</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>誰でも参加可</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>anyone joins</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>emp_ui_team_closed</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>リーダーが承認</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>the leader answers</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>emp_ui_team_online</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>オンライン</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>emp_ui_team_offline</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>オフライン</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>offline</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>emp_ui_team_leader_tag</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>（リーダー）</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>(leader)</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>emp_ui_team_lands</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>土地</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>emp_ui_team_no_land</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>まだ土地がありません。</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>No land yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>emp_ui_team_others</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>他のチーム</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>Other teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>emp_ui_team_line</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>{0}  リーダー {1}  {2}人  {3}</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>{0}  led by {1}  {2} members  {3}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Server info page: message of the day and rules, personal friends and ignore lists, admin announcements and restart warnings
Texts travel with the world's rules (keys 139-140) from ElinMP/motd.txt and rules.txt; a one-line log notice for a text the player has not read; an ignored player's chat bubbles and whispers are dropped on the player's side; admins say/restart through AdminCommandDelta; server notices use MsgSayDelta.Notice.

Not run in game (no game access for this worker): bench/server_info_check.py written, compile checked.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D634"/>
+  <dimension ref="A1:D659"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11297,6 +11297,431 @@
         </is>
       </c>
     </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>emp_ui_tab_info</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>サーバー情報</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Server</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>emp_info_notice</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>サーバーのルールは Elin Together メニューで読めます。</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Read the server rules in the Elin Together menu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>emp_info_motd</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>今日のお知らせ</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Message of the day</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>emp_info_rules</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>サーバーのルール</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Server rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>emp_info_none</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>ホストはまだ何も書いていません。</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>The host has not written anything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>emp_info_edit_motd</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>お知らせを書く</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Write the message of the day</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>emp_info_edit_rules</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>ルールを書く</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Write the rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>emp_info_reload</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>ファイルを再読込して全員に送る</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Reload the files and send to everyone</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>emp_info_files</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>ホストの ElinMP フォルダの motd.txt と rules.txt を直接編集しても構いません。入力欄では | が改行になります。</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>You can also edit motd.txt and rules.txt in the host's ElinMP folder. In the input box, a | is a line break.</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>emp_info_announce</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>全員へのお知らせ</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Announcements</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>emp_info_say</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>全員にお知らせを送る</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Tell everyone</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>emp_info_restart_10</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>再起動の予告（10分前）</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Warn of a restart (10 min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>emp_info_restart_cancel_button</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>予告を取り消す</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Cancel the warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>emp_info_restart</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>サーバーは{0}分後に再起動します。</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>The server restarts in {0} min.</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>emp_info_restart_cancel</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>サーバーの再起動は取り消されました。</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>The restart is cancelled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>emp_info_friends</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>フレンド</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>emp_info_friend_online</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>{0}（オンライン）  {1}</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>{0} (online)  {1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>emp_info_friend_offline</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>{0}（オフライン）</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>{0} (offline)</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>emp_info_friends_none</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>フレンドはいません。プレイヤー一覧のメニューから追加できます。</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>No friends yet. Add one from a player's menu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>emp_info_ignored</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>無視リスト</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Ignored players</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>emp_info_ignored_note</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>このゲームだけで、相手の発言とささやきが非表示になります。相手には知らされません。</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Their chat and whispers are hidden in your game only. They are told nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>emp_ui_ignore</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>無視する</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Ignore</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>emp_ui_unignore</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>無視をやめる</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Stop ignoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>emp_ui_friend</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>フレンドに追加</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Add friend</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>emp_ui_unfriend</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>フレンドから外す</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Remove friend</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Team leaders manage their team: rename, kick, promote, disband, invitations (host box, off by default), team size cap and found wait
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D650"/>
+  <dimension ref="A1:D685"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11569,6 +11569,615 @@
         </is>
       </c>
     </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_team_leaders</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>チームのリーダーが自分のチームを管理する</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Team leaders manage their team</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_team_leaders</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>リーダーはチームページで名前変更、メンバーの追放、リーダーの委譲、解散、プレイヤーの招待ができます。チームの人数とチーム作成の間隔にも上限があります。オフ：プレイヤー一覧の作成・参加・脱退とリーダーの承認のみ。</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>The leader can rename the team, put a member out, hand the team over, end it and invite players from the Team page. A team's size and how often a player founds a team are limited. Off: only found, join, leave and the leader's yes or no from the list of players.</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_team_max_size</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>チームの最大人数</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>Players per team</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_team_max_size</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>5人：チームは5人まで。
+10人：10人まで。
+20人：20人まで。
+50人：50人まで。
+制限なし：人数の上限なし。</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>5: a team holds up to 5 players.
+10: up to 10.
+20: up to 20.
+50: up to 50.
+No limit: any number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_team_max_size_5</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>5人</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_team_max_size_10</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>10人</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_team_max_size_20</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>20人</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_team_max_size_50</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>50人</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_team_max_size_0</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>制限なし</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>No limit</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_team_found_cooldown</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>チーム再作成までの待ち時間</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Wait before founding another team</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_team_found_cooldown</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>なし：すぐに別のチームを作れます。
+5分：5分待ちます。
+30分：30分待ちます。
+60分：60分待ちます。</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>None: a player may found another team at once.
+5 minutes: it waits 5 minutes.
+30 minutes: 30.
+60 minutes: 60.</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_team_found_cooldown_0</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>なし</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_team_found_cooldown_5</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>5分</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>5 minutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_team_found_cooldown_30</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>30分</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>30 minutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_team_found_cooldown_60</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>60分</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>60 minutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>emp_ui_team_manage</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>リーダーの操作</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Leader's choices</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>emp_ui_team_rename</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>チーム名を変更</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>Rename the team</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>emp_ui_team_rename_ask</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>チームの新しい名前</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>New name of the team</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>emp_ui_team_promote</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>リーダーにする</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>Make leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>emp_ui_team_kick</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>チームから外す</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>Put out of the team</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>emp_ui_team_invite</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>{0}を招待</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>Invite {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>emp_ui_team_invited_line</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>{0}を招待済み（返事待ち）</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>{0} is invited (waiting for an answer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>emp_ui_team_disband</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>チームを解散</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>Disband the team</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>emp_ui_team_disband_confirm</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>{0}を解散しますか？メンバーは放浪者に戻り、土地は誰のものでもなくなります。</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>Disband {0}? Its members become Wanderers and its lands nobody's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>emp_ui_team_invite_title</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>招待</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>Invitation</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>emp_ui_team_invite_line</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>{0}（リーダー：{1}）があなたを招待しています。</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>{0} (leader: {1}) invites you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>emp_ui_team_invite_accept</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>招待を受ける</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>Accept</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>emp_ui_team_invite_refuse</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>断る</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>Refuse</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>emp_team_kicked</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>あなたは{0}から外されました。</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>You were put out of {0}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>emp_team_promoted</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>あなたが{0}のリーダーになりました。</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>You now lead {0}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>emp_team_disbanded</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>{0}は解散しました。</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>{0} was disbanded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>emp_team_invited</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>{1}が{0}に招待しています。チームページで答えてください。</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>{1} invites you to {0}. Answer on the Team page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>emp_team_invite_refused</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>{0}は招待を断りました。</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>{0} refused your invitation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>emp_team_full</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>{0}はいっぱいです。</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>{0} is full.</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>emp_team_found_wait</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>別のチームを作るにはあと{0}分待ってください。</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Wait {0} more minutes before founding another team.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Land rules: a level for the team and one for others per land, Teams.Allowed replaces the fixed test (host box, off = today)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D685"/>
+  <dimension ref="A1:D694"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -12178,6 +12178,159 @@
         </is>
       </c>
     </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_land_rules</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>土地ごとのルール</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>Rules for each land</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_land_rules</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>チームのリーダーは土地ごとに、自分のチームとそれ以外の人が何をできるか（立入禁止、見学、見学と使用、建築）を決めます。「拠点をチームが所有」が必要です。オフ：土地は従来どおり、チームは建築でき、他の人は見学のみ。</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>A team's leader sets, for each of its lands, what its own team and everyone else may do there: closed, visit, visit and use, or build. Needs "Team ownership of bases". Off: a land is as before, its team builds and others visit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>emp_ui_team_rule_0</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>立入禁止</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>emp_ui_team_rule_1</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>見学</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>Visit</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>emp_ui_team_rule_2</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>見学と使用</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Visit and use</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>emp_ui_team_rule_3</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>建築</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>emp_ui_team_rule_mine</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>この土地で：自分のチーム</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>On this land: my team</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>emp_ui_team_rule_others</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>この土地で：それ以外の人</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>On this land: everyone else</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>emp_ui_team_land_line</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>{0}：チーム＝{1}、他の人＝{2}</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>{0}: team = {1}, others = {2}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Container access log; moderator, freeze and jail
Host box "Container access log": who put or took what per container of a land (and the bank and delivery boxes), last 50 entries in the save, read from the container's right-click menu by the land's team and admins, and from the Elin Together menu by admins (ContainerLogRequest 1210 / ContainerLogAnswer 1211).
Host box "Moderators, freeze and jail": a moderator who only mutes, unmutes and kicks; freeze = the game's paralysis kept on the player's character; jail = sent to the zone an admin chose (TeamSpawnDelta) and frozen. Per-player rollback not done (design question).
Not run in the game: written without access to it; bench/workerA_check.py is untested.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D634"/>
+  <dimension ref="A1:D652"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11297,6 +11297,312 @@
         </is>
       </c>
     </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>emp_container_log</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>アクセスログ</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Access log</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>emp_container_logs_title</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>コンテナのアクセスログ</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Container access logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>emp_container_log_empty</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>(まだ記録なし)</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>(nothing recorded yet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>emp_container_log_put</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>{0}  {1} が {3} を {2} 個入れた</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>{0}  {1} put {2} x {3}</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>emp_container_log_took</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>{0}  {1} が {3} を {2} 個取った</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>{0}  {1} took {2} x {3}</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>emp_ui_container_logs</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>コンテナのアクセスログ</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Container logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>emp_ui_freeze</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>凍結</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Freeze</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>emp_ui_unfreeze</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>凍結解除</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Unfreeze</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>emp_ui_jail</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>投獄</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Jail</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>emp_ui_set_jail</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>ここを牢屋にする</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Use this zone as the jail</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>emp_ui_make_mod</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>モデレーターにする</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Make moderator</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>emp_ui_unmake_mod</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>モデレーター解除</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Remove moderator</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>emp_ui_mod_tag</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>[モデレーター]</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>[moderator]</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>emp_ui_frozen_tag</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>[凍結中]</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>[frozen]</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_container_log</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>コンテナのアクセスログ</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>Container access log</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_container_log</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>プレイヤーやチームの土地にあるコンテナ(銀行と宅配ボックスも)ごとに、誰がいつ何を入れた・取ったかを直近50件ホストが記録します。土地のチームと管理者がコンテナの右クリックメニューから読めます。オフ:記録も表示もしません。</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>The host records, per container of a player's or team's land (and the bank and delivery boxes), who put or took what and when (last 50 entries). The land's team and the admins read it from the container's right-click menu. Off: nothing is recorded or shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_admin_extras</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>モデレーター・凍結・投獄</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Moderators, freeze and jail</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_admin_extras</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>ホストが任命するモデレーターはミュートとキックだけ可能。管理者は凍結(解除まで行動不能)と投獄(指定マップへ送って凍結)ができます。ホストと他の管理者は対象外。オフ:これらの命令は拒否されます。</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>Moderators the host appoints can only mute and kick. Admins can freeze (no action until released) and jail (sent to the chosen map and frozen). Never the host or another admin. Off: these orders are refused.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Closed lands: entry refused on the lease and on the host's own travel, never trapping (30 s grace then moved out, TeamEvictDelta 1200)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D694"/>
+  <dimension ref="A1:D696"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -12331,6 +12331,40 @@
         </is>
       </c>
     </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>emp_land_closed</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>この土地はあなたに閉ざされています。</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>This land is closed to you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>emp_land_leave_notice</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>{0}はあなたに閉ざされています。{1}秒後に外へ移動します。</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>{0} is closed to you. You will be moved out in {1} seconds.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Offline protection: a land option closes it to others while no member of its team is online
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D696"/>
+  <dimension ref="A1:D698"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -12365,6 +12365,40 @@
         </is>
       </c>
     </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>emp_ui_team_rule_offline</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>チームの誰もオンラインでない間は他の人に閉ざす</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Closed to others while no member of the team is online</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>emp_ui_team_rule_offline_tag</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>（留守中は閉鎖）</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>(closed while away)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Abandoned land: a team away for N real days loses its claim (host box, default 30 days), lands-per-team cap
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D698"/>
+  <dimension ref="A1:D716"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -12399,6 +12399,330 @@
         </is>
       </c>
     </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_land_abandon</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>放置された土地を手放す</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>Abandoned land</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_land_abandon</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>チームの誰も現実の日数のあいだゲームに入らなかった場合、そのチームは土地の所有権を失い、土地は誰のものでもなく全員に開放されます。オフ：チームは長く留守にしても土地を保持します。</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>A team none of whose members came into the game for the days set below loses its claim on its lands: they become nobody's and open to everyone. Off: a team keeps its lands however long it is away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_abandon_days</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>土地を手放すまでの日数</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Days away before the land is lost</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_abandon_days</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>7日：チームが1週間来なかった場合。
+14日：2週間。
+30日：30日間。
+60日：60日間。
+90日：90日間。</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>7 days: the team was away a week.
+14 days: two weeks.
+30 days: thirty days.
+60 days: sixty days.
+90 days: ninety days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_abandon_days_7</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>7日</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>7 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_abandon_days_14</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>14日</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>14 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_abandon_days_30</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>30日</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>30 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_abandon_days_60</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>60日</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>60 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_abandon_days_90</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>90日</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>90 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_lands_per_team</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>チームあたりの土地の上限</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>Lands per team</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_lands_per_team</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>1：チームは土地を1つまで。
+2：2つまで。
+3：3つまで。
+5：5つまで。
+10：10まで。
+制限なし：上限なし。</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>1: a team claims one land.
+2: two.
+3: three.
+5: five.
+10: ten.
+No limit: any number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_lands_per_team_1</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>1つ</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_lands_per_team_2</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>2つ</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_lands_per_team_3</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>3つ</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_lands_per_team_5</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>5つ</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_lands_per_team_10</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_lands_per_team_0</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>制限なし</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>No limit</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>emp_team_land_cap</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>あなたのチームはすでに{0}つの土地を持っています。これ以上は主張できません。</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>Your team already holds {0} lands. It cannot claim more.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Several lands per tile, step 1: a deed read on an occupied tile makes another plot there
Host box "Several lands per tile" (off by default, rules key 144, SiblingLandDelta 1225). TraitDeed.OnRead on the world
map on a tile that holds a land asks, then the host makes a second wild field at the same x,y (reused if one is
waiting), the reader steps in and reads the deed again: the game's own claim, so the lands-per-team cap and the Teams
rules apply as always. A guest asks the host (read again there like BaseRelocateDelta), alone on its world map too.
Not run in game (no game access in this worktree); the bench script comes with the last step.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D762"/>
+  <dimension ref="A1:D765"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -13505,6 +13505,57 @@
         </is>
       </c>
     </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_sibling_lands</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>複数の土地を1マスに</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>Several lands per tile</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_sibling_lands</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>世界地図の1マスに、別々のチームの土地を複数置けます。すでに土地があるマスで土地証書を読むと、同じマスに別の区画ができます。複数の土地があるマスに入ると、入る土地を選ぶ一覧が出ます。「拠点をチームが所有」が必要です。オフ：1マスにつき土地は1つ。</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>Lands of different teams may share one world-map tile. A deed read on a tile that already holds a land makes another plot there, and stepping onto a tile with several lands lists them to pick one. Needs "Team ownership of bases". Off: one land per tile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>emp_sibling_ask</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>この場所にはすでに土地があります。同じマスに別の区画を作りますか？その区画に入り、もう一度証書を読んで主張します。</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>This tile already holds a land. Make another plot on it? You step into the plot and read the deed again to claim it.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Several lands per tile, step 2: walking onto a tile with two lands or more lists them
Player.EnterLocalZone takes the first zone at the tile; with the host box on and 2+ lands there, a list opens (team name,
land, what the land lets this player do; a closed one greyed and refusing) and the choice is the zone itself, so the
travel and the lease request already carry its uid. The host reads it again with Teams.EntryDenied (LeaseZone) and for its
own travel, as for any land. One land, or the box off: the game as it was. Not run in game.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D765"/>
+  <dimension ref="A1:D766"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -13556,6 +13556,23 @@
         </is>
       </c>
     </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>emp_sibling_pick</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>どの土地に入りますか</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>Which land to enter</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Server avatar step 1: the stand-in, Exchange() out of TakeOverPc, forward migration at -empserver load
- Exchange(mine, formerOwner, me): the swap of who is the local character, extracted unchanged from TakeOverPc (classic hosting and the save depot behave as before)
- ServerAvatar (Helper), table server_avatar in the save, setting ServerAvatar (on, used only under -empserver, row in the Repair group, EN/JP/CN texts)
- at -empserver load the owner's character is exchanged for a hidden stand-in once, with a backup before the first exchange (no backup = no exchange); the session opens only after (ServerAvatar.Settled)
- bench/avatar_suite.py: AV0 server identity, AV1 exchange and backup, AV2 the owner joins with its own character

Not run here (no game): see the bench script.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D680"/>
+  <dimension ref="A1:D682"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -12079,6 +12079,40 @@
         </is>
       </c>
     </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_server_avatar</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>サーバーは誰も操作しない</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>Server plays no character</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_server_avatar</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>専用サーバー(-empserver)は誰も操作しません。セーブの持ち主のキャラクターは、そのSteam IDに結びついた通常のプレイヤーキャラになり(他の参加者と同じく参加します)、サーバー自身は隠れた無敵の代役を使います。オフ:持ち主のキャラクターは今までどおり拠点に置かれます。メニューから開始したゲームには影響しません。</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>A dedicated server (-empserver) plays no character: the save owner's character becomes an ordinary player character tied to its Steam id (it joins like any guest), and the server's own player is a hidden, untouchable stand-in. Off: the owner's character stays planted at the base as before. Has no effect on a game hosted from the menu.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hidden server: host box "Play as a guest of a hidden server (beta)" starts the world in a hidden -empserver game and joins it; parent-pid watchdog, server.stop on quit, lobby id file for invites, config.txt untouched by a server
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D768"/>
+  <dimension ref="A1:D779"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -13607,6 +13607,193 @@
         </is>
       </c>
     </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_hidden_server</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>隠しサーバーのゲストとして遊ぶ（ベータ）</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>Play as a guest of a hidden server (beta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_hidden_server</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>「サーバー開始」でワールドをこのPC上の隠れた2つ目のElinで動かし、自分のゲームは他のプレイヤーと同じように参加します。ホストキャラクターがなくなり、体験が友達と同じになります。空きメモリが約2GB必要です。2分以内に起動しない場合は従来どおりホストします。Windowsのみ。</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>"Start Server" runs your world in a second, hidden Elin on this PC and your own game joins it like any other player: no host character, you live what your friends live. Needs about 2 GB of free memory; if the hidden game is not up in 2 minutes, the world is hosted as before. Windows only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>emp_hidden_starting</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>ワールドを起動しています...</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>Starting your world...</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>emp_hidden_fallback</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>隠しサーバーは使えませんでした（{0}）。ワールドは従来の方法で開放します。</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>The hidden server could not be used ({0}): your world is hosted the usual way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>emp_hidden_why_save</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>ここではゲームを保存できません</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>the game cannot save here</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>emp_hidden_why_mutex</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>ゲームが多重起動の制限を解除できませんでした</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>the game could not lift its one-instance lock</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>emp_hidden_why_launch</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>隠しゲームを起動できませんでした</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>the hidden game could not be started</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>emp_hidden_why_exit</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>隠しゲームが途中で終了しました</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>the hidden game stopped on its own</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>emp_hidden_why_timeout</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>2分以内に起動しませんでした</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>it was not up in 2 minutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>emp_hidden_why_cancel</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>起動を中止しました</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>starting was cancelled</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>emp_travel_hidden_owner</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>隠しサーバーで遊んでいる間は、一人で別のマップを管理できません。仲間と一緒に移動してください。</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>While you play on a hidden server you cannot hold a map on your own: travel with the others.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hidden server identity: the server has a reserved id in Release too, listens on 127.0.0.1 when hidden, the loopback seat of its own account is the owner's only with the owner token (first handshake), is an admin, holds no map and opens no listener; host-identity sites use ServerAvatar.HostUser
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D779"/>
+  <dimension ref="A1:D780"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -13794,6 +13794,23 @@
         </is>
       </c>
     </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>emp_dc_owner_seat</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>この席は隠しサーバーの所有者専用です。</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>This seat belongs to the owner of this hidden server.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Team boxes: copies told every 0.2 s; the Team tab shows the team bank's gold
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D780"/>
+  <dimension ref="A1:D781"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -13811,6 +13810,23 @@
         </is>
       </c>
     </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>emp_ui_team_bank</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>チームの銀行：{0}</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Team bank: {0} gold</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Team boxes: the personal, team and old-world bank windows open side by side, each with its title
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D781"/>
+  <dimension ref="A1:D786"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,6 +467,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -13827,6 +13828,91 @@
         </is>
       </c>
     </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>emp_box_own_bank</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>個人の銀行</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Personal bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>emp_box_team_bank</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>チームの銀行: {0}</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>Team bank: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>emp_box_world_bank</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>共有の銀行(旧ワールド)</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>Shared bank (old world)</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>emp_box_own_delivery</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>個人の配達ボックス</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>Personal delivery box</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>emp_box_world_delivery</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>共有の配達ボックス(旧ワールド)</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>Shared delivery box (old world)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Multiplayer hub: HUD button in the main-menu hotbar, polished window
A vanilla HotItemLayer in hotbar 2 (postfix on ResetHotbar, prefix on HotItemLayer.OnClick) opens/closes the layer
for host and guests alike; the icon is two of the game's own putit sprites, built at runtime. The window gets a
caption icon, a sprite and a tooltip per tab, and a fixed size.

Not run in game (compile only); bench/hub_button_check.py covers it.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D786"/>
+  <dimension ref="A1:D793"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -13913,6 +13913,125 @@
         </is>
       </c>
     </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>LayerElinTogether</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>マルチプレイ</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>Multiplayer</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_session</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>接続中のゲームと参加者</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>The game you are in and who is playing</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_team</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>チームの所属と権限</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>Teams: who is in which, and what a leader may do</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_server</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>ホストのワールドルール</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>The world rules set by the host</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_info</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>サーバーの案内とルール</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>Server message and rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_lobby</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>ゲームの作成・参加</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>Host a game or find one to join</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_client</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>自分用の設定</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>Your own settings</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hub step 3: EmpUi pieces (player row, setting rows, card, chip, empty state) and a debug demo layer
Reusable vanilla-looking UI parts for the multiplayer hub, built on the game's own prefabs (headers, texts,
Tag General chip, Portrait, context menu) and sprites. Not used by any tab yet. emp.ui_demo (DEBUG) opens a
layer that shows each piece.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D786"/>
+  <dimension ref="A1:D787"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -13913,6 +13913,23 @@
         </is>
       </c>
     </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>emp_ui_set_by_host</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>ホストが設定</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>Set by the host</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
World rules page: banner, preset cards, search, collapsible groups, folded advanced rows, changed dot and revert
Read-only for a friend (same data path), one summary line when the host changes several rules within a second.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D786"/>
+  <dimension ref="A1:D800"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6962,12 +6962,12 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>その他の設定は Elin Together のウィンドウ（「ワールドのルール」タブ）にあります。</t>
+          <t>さらに{0}件を表示</t>
         </is>
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>More options in the Elin Together window (World rules tab).</t>
+          <t>Show {0} more</t>
         </is>
       </c>
     </row>
@@ -13913,6 +13913,244 @@
         </is>
       </c>
     </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_banner_host</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>あなたが決めます</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>You decide</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_banner_guest</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>{0}が設定</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>Set by {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_search</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>ルールを検索</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>Search the rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_nomatch</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>一致するルールはありません。</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>No rule matches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_preset_current</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>現在</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_diff_title</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>おすすめとの違い（{0}件）</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>Differs from Recommended ({0})</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_diff_all</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>すべて表示（{0}）</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>Show all {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_fewer</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>表示を減らす</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>Show fewer</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_revert</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>元に戻す</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>Revert</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_needs</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>「{0}」が必要です</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>Needs: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_needs_off</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>「{0}」をオフにする必要があります</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>Needs this off: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_needs_notofficial</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>公式サーバーでは使えません</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>Not available on the official server</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_needs_other</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>他のルールがオンである必要があります</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>Needs another rule to be on</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>emp_ui_rules_changed_many</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>ホストが{0}件のルールを変更しました：{1}</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>The host changed {0} rules: {1}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hub step 7: Server info notes, My settings cards with friends and ignored, Help page, World rules tab for guests
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D808"/>
+  <dimension ref="A1:D837"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -680,12 +680,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>サーバー</t>
+          <t>ワールドのルール</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Server</t>
+          <t>World rules</t>
         </is>
       </c>
     </row>
@@ -1417,12 +1417,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>クライアント設定</t>
+          <t>自分の設定</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Client settings</t>
+          <t>My settings</t>
         </is>
       </c>
     </row>
@@ -1434,12 +1434,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>クライアント</t>
+          <t>自分の設定</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>My settings</t>
         </is>
       </c>
     </row>
@@ -11429,7 +11429,7 @@
       </c>
       <c r="D642" t="inlineStr">
         <is>
-          <t>The host has not written anything.</t>
+          <t>The host hasn't written anything yet.</t>
         </is>
       </c>
     </row>
@@ -11492,12 +11492,12 @@
       </c>
       <c r="C646" t="inlineStr">
         <is>
-          <t>ホストの ElinMP フォルダの motd.txt と rules.txt を直接編集しても構いません。入力欄では | が改行になります。</t>
+          <t>ホストの ElinMP フォルダの motd.txt と rules.txt を直接編集しても構いません。</t>
         </is>
       </c>
       <c r="D646" t="inlineStr">
         <is>
-          <t>You can also edit motd.txt and rules.txt in the host's ElinMP folder. In the input box, a | is a line break.</t>
+          <t>You can also edit motd.txt and rules.txt in the host's ElinMP folder.</t>
         </is>
       </c>
     </row>
@@ -13972,12 +13972,12 @@
       </c>
       <c r="C790" t="inlineStr">
         <is>
-          <t>ホストのワールドルール</t>
+          <t>ホストが決めたワールドのルール（ゲストは閲覧のみ）</t>
         </is>
       </c>
       <c r="D790" t="inlineStr">
         <is>
-          <t>The world rules set by the host</t>
+          <t>The world's rules set by the host (guests read them)</t>
         </is>
       </c>
     </row>
@@ -14023,12 +14023,12 @@
       </c>
       <c r="C793" t="inlineStr">
         <is>
-          <t>自分用の設定</t>
+          <t>自分だけの設定、フレンド、無視リスト</t>
         </is>
       </c>
       <c r="D793" t="inlineStr">
         <is>
-          <t>Your own settings</t>
+          <t>Your own options, friends and ignored players</t>
         </is>
       </c>
     </row>
@@ -14284,6 +14284,499 @@
       <c r="D808" t="inlineStr">
         <is>
           <t>The host changed {0} rules: {1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>emp_tab_info</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>サーバー</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>Server</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>emp_ui_tab_help</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>ヘルプ</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>Help</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>emp_tab_help</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>ヘルプ</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>Help</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_help</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>使い方、バージョン、バグ報告</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>How it works, version and bug report</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>emp_info_none_host</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>まだ何も書いていません。参加者全員に表示されます。</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>Nothing written yet. Every player can read it here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>emp_info_write</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>書く</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>Write one</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>emp_info_edit</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>鉛筆で編集</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>Edit (pencil)</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>emp_info_save</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>保存して全員に送る</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>Save and send to everyone</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>emp_info_cancel</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>キャンセル</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>Cancel</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>emp_hub_change</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>変更</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>emp_hub_online</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>オンライン: {0}</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>Online: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>emp_hub_offline</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>オフライン</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>emp_help_hosting_t</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>ゲームを開く</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>Hosting a game</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>emp_help_hosting</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>「プレイ」ページで「このゲームをホストする」を押すと、今のセーブが友達に公開されます。ルールは「ワールドのルール」で決めます。</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>On the Play page, press Host this game: your current save opens to friends. You decide the rules on the World rules page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>emp_help_joining_t</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>友達のゲームに参加する</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Joining a friend</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>emp_help_joining</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>「プレイ」ページで友達か公開サーバーを選ぶだけです。あなたのキャラクターはそのワールドに保存されます。</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>Pick a friend or a public server on the Play page. Your character is kept in that world.</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>emp_help_teams_t</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>チーム</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>Teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>emp_help_teams</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>チームは一緒に行動し、土地や所持品を分け合います。リーダーが仲間を招待・追放できます。ホストが有効にした場合のみ使えます。</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>A team travels together and shares lands. Its leader can invite and remove members. Available when the host turns teams on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>emp_help_lands_t</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>土地</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>emp_help_lands</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>土地は、入れる人と触れる人が決まっています。チームの銀行と配達箱は、チーム全員で使えます。</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>Each land says who may enter and who may touch things. The team bank and delivery box are shared by the whole team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>emp_help_trading_t</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>取引</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>Trading</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>emp_help_trading</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>プレイヤー一覧のメニューから「取引」を選ぶと、相手と品物やお金を交換できます。</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>Choose Trade in a player's menu to swap items and money with them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>emp_help_duels_t</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>決闘</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>Duels</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>emp_help_duels</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>プレイヤーのメニューから決闘を申し込めます。相手が受けた時だけ始まります。</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>Challenge a player from their menu. It starts only if they accept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>emp_help_about</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>このMODについて</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>About</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>emp_help_version</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Elin Together（独立版）{0}</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>Elin Together (independence) {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>emp_help_about_desc</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>最新版、不具合の報告、ソースコードはGitHubにあります。</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>The latest version, bug reports and the source are on GitHub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>emp_help_github</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>GitHubを開く</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>Open GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>emp_help_report</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>不具合を報告する</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>Report a bug</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hub step 4: Play and Players pages (EmpUi rows, cards, chips), replacing the Lobby and Session tabs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D808"/>
+  <dimension ref="A1:D836"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -14287,6 +14287,482 @@
         </is>
       </c>
     </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>emp_ui_tab_play</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>プレイ</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>Play</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>emp_ui_tab_players</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>プレイヤー</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>Players</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_play</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>ゲームを開く・参加・退出</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>Host, join or leave a game</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_players</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>参加中のプレイヤーと操作</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>Who is playing, and what you can do with them</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>emp_ui_play_connected</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>接続中</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>Connected</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>emp_ui_play_reconnecting</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>再接続中...</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>Reconnecting...</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>emp_ui_play_world</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>{0}のワールド</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>{0}'s world</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>emp_ui_play_host_line</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>ホスト: {0}</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>Host: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>emp_ui_play_players_line</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>プレイヤー: {0}人</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>Players: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>emp_ui_play_where</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>現在地: {0}</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>Now in: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>emp_ui_play_host_title</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>このゲームをホストする</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>Host this game</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>emp_ui_play_host_desc</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>このワールドを友達に開放します。友達はSteamか下の公開リストから参加できます。</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>Open this world to your friends. They join from Steam or from the public list below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>emp_ui_play_host_title_screen</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>先にワールドを読み込み、このページで「サーバー開始」を押してください。</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>Load your world first, then open this page and press Start server.</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>emp_ui_play_host_depot</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>共有ワールドはオンラインに保管されています。ワンクリックで引き継いでホストできます。</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>The shared world is kept online. Take it over and host it in one click.</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>emp_ui_play_join_title</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>友達に参加する</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Join a friend</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>emp_ui_play_join_desc</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Steamの招待を受けるか、アドレスでサーバーに参加します。</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>Accept a Steam invite from a friend, or join a server by its address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>emp_ui_play_join_ingame</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>参加するにはタイトル画面に戻ってください。</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>Go back to the title screen to join a game.</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>emp_ui_play_public_title</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>公開サーバー</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>Public servers</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>emp_ui_play_searching</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>ゲームを探しています...</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Looking for games...</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>emp_ui_play_none</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>今は公開されているゲームがありません。</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>No public game right now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>emp_ui_players_title</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>プレイヤー ({0})</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>Players ({0})</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>emp_ui_player_detail</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>{0}、レベル{1}</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>{0}, level {1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>emp_ui_player_host</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>ホスト</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>emp_ui_player_you</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>(あなた)</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>(you)</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>emp_ui_act_whisper</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>ささやく</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>Whisper</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>emp_ui_players_alone</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>ここにはあなた一人です。</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>You're alone here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>emp_ui_players_alone_btn</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>友達を招待</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>Invite a friend</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>emp_ui_players_go_play</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>ゲームを開く・参加する</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>Host or join a game</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hub step 5: Team and Lands pages
Team: header with the team name and an "Open to all" chip, member rows with portraits and a crown, leader tools in one card (greyed with a reason for non-leaders, "..." on a member row for Make leader / Remove from team), joining toggle (TeamAsk.SetOpen), requests and invitations as accept/refuse rows, and a "Teams are off in this world" empty state with a host-only "Turn on" that opens the World rules tab at the Teams row. Lands: a card per land with the land-rule drop-downs, offline protection and container log, then the team bank and delivery box with the game's item icons. Both tabs are always in the window.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D808"/>
+  <dimension ref="A1:D839"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -12628,12 +12628,12 @@
       </c>
       <c r="C712" t="inlineStr">
         <is>
-          <t>リーダーの操作</t>
+          <t>リーダーツール</t>
         </is>
       </c>
       <c r="D712" t="inlineStr">
         <is>
-          <t>Leader's choices</t>
+          <t>Leader tools</t>
         </is>
       </c>
     </row>
@@ -12701,7 +12701,7 @@
       </c>
       <c r="D716" t="inlineStr">
         <is>
-          <t>Put out of the team</t>
+          <t>Remove from team</t>
         </is>
       </c>
     </row>
@@ -14287,6 +14287,533 @@
         </is>
       </c>
     </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>emp_ui_tab_lands</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>土地</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>emp_tab_lands</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>土地</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_lands</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>チームの土地：ルール、留守中の保護、銀行と配達ボックス</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>The team's lands: rules, protection while away, bank and delivery box</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>emp_ui_team_chip_open</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>誰でも参加可</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>Open to all</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>emp_ui_team_chip_closed</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>リーダーが承認</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>Leader approves</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>emp_ui_team_leader_line</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>リーダー：{0}　メンバー{1}人</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>Leader: {0}  ·  {1} members</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>emp_ui_team_detail</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Lv {0}、{1}</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>Lv {0}, {1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>emp_ui_team_crown</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>リーダー</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>emp_ui_team_off</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>このワールドではチームは無効です。</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>Teams are off in this world.</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>emp_ui_team_off_guest</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>このワールドではチームは無効です。ホストだけがオンにできます。</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>Teams are off in this world. Only the host can turn them on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>emp_ui_team_unplugged</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>チームはマルチプレイの中で使えます。プレイページでホストするか参加してください。</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>Teams work in a multiplayer game. Host or join one on the Play page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>emp_ui_team_turn_on</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>オンにする</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>Turn on</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>emp_ui_team_requests</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>参加の申請</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>Requests to join</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>emp_ui_team_asks_row</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>{0}が参加を希望しています</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>{0} asks to join</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>emp_ui_team_tools_leader_only</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>リーダーだけが使えます。</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Only the leader of the team can use these.</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>emp_ui_team_tools_host_off</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>ホストがこのワールドでリーダーの操作をオフにしています。</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>The host turned leader tools off in this world.</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>emp_ui_team_leader_only_chip</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>リーダーのみ</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>Leader only</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>emp_ui_team_joining</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>誰でも参加可</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>Anyone may join</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>emp_ui_team_joining_desc</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>オフにすると、リーダーが申請ごとに答えます。</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Off: the leader answers each request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>emp_ui_team_invite_any</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>プレイヤーを招待</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>Invite a player</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>emp_ui_team_invite_none</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>招待できるチームなしのプレイヤーはいません。</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>No one in the game without a team to invite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>emp_ui_land_where</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>場所：{0}</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>In {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>emp_ui_land_none</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>まだ土地がありません。野原で土地の権利書を読むと手に入ります。</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>No land yet. Read a land deed on a field to claim one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>emp_ui_land_noteam</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>土地を持つには、まずチームを作るか参加してください。</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>Found or join a team to hold land.</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>emp_ui_land_rules_off</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>このワールドでは土地のルールはオフです。</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>Land rules are off in this world.</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>emp_ui_land_leader_decides</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>ルールを変えられるのはリーダーだけです。</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>Only the leader changes these.</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>emp_ui_land_boxes</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>銀行と配達ボックス</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>Bank and delivery box</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>emp_ui_land_team_bank</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>チームの銀行</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>Team bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>emp_ui_land_bank_line</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>{0}ゴールド、品物{1}個</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>{0} gold, {1} items</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>emp_ui_land_delivery</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>あなたの配達ボックス</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>Your delivery box</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>emp_ui_land_items</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>品物{0}個</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>{0} items</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hub: wording pass (sentence case, same terms: host/guest/team/land), EN/JP/CN in sync, texts for the new empty-state buttons
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D896"/>
+  <dimension ref="A1:D899"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2589,12 +2589,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>これはホストのルールです。変更はすぐ全員に反映されます。</t>
+          <t>これはホストのルールです。変更はプレイ中の全員にすぐ反映されます。</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>These are the host's rules. Changes apply to everyone at once.</t>
+          <t>These are the host's rules. Changes apply at once to every player.</t>
         </is>
       </c>
     </row>
@@ -7064,12 +7064,12 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>ワールドを置いておく場所で、誰でもホストになれます。一緒に遊ぶだけなら必要ありません。</t>
+          <t>ワールドを置いておく場所で、どのプレイヤーもホストになれます。一緒に遊ぶだけなら必要ありません。</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>Where the world is kept so that any of you can host it. Not needed to play together.</t>
+          <t>Where the world is kept so that any player can host it. Not needed to play together.</t>
         </is>
       </c>
     </row>
@@ -11361,7 +11361,7 @@
       </c>
       <c r="D638" t="inlineStr">
         <is>
-          <t>Server</t>
+          <t>Server info</t>
         </is>
       </c>
     </row>
@@ -11373,12 +11373,12 @@
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>サーバーのルールは Elin Together メニューで読めます。</t>
+          <t>サーバーのルールはマルチプレイメニューで読めます。</t>
         </is>
       </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>Read the server rules in the Elin Together menu.</t>
+          <t>Read the server rules in the Multiplayer menu.</t>
         </is>
       </c>
     </row>
@@ -12764,12 +12764,12 @@
       </c>
       <c r="C720" t="inlineStr">
         <is>
-          <t>{0}を解散しますか？メンバーは放浪者に戻り、土地は誰のものでもなくなります。</t>
+          <t>{0}を解散しますか？メンバーは放浪者に戻り、土地は持ち主がいなくなります。</t>
         </is>
       </c>
       <c r="D720" t="inlineStr">
         <is>
-          <t>Disband {0}? Its members become Wanderers and its lands nobody's.</t>
+          <t>Disband {0}? Its members become Wanderers and its lands lose their owner.</t>
         </is>
       </c>
     </row>
@@ -12854,7 +12854,7 @@
       </c>
       <c r="D725" t="inlineStr">
         <is>
-          <t>You were put out of {0}.</t>
+          <t>You were removed from {0}.</t>
         </is>
       </c>
     </row>
@@ -13989,12 +13989,12 @@
       </c>
       <c r="C791" t="inlineStr">
         <is>
-          <t>サーバーの案内とルール</t>
+          <t>ホストからの案内とルール</t>
         </is>
       </c>
       <c r="D791" t="inlineStr">
         <is>
-          <t>Server message and rules</t>
+          <t>The host's message and rules</t>
         </is>
       </c>
     </row>
@@ -14295,12 +14295,12 @@
       </c>
       <c r="C809" t="inlineStr">
         <is>
-          <t>サーバー</t>
+          <t>サーバー情報</t>
         </is>
       </c>
       <c r="D809" t="inlineStr">
         <is>
-          <t>Server</t>
+          <t>Server info</t>
         </is>
       </c>
     </row>
@@ -15558,7 +15558,7 @@
       </c>
       <c r="D883" t="inlineStr">
         <is>
-          <t>Anyone may join</t>
+          <t>Open to all</t>
         </is>
       </c>
     </row>
@@ -15570,12 +15570,12 @@
       </c>
       <c r="C884" t="inlineStr">
         <is>
-          <t>オフにすると、リーダーが申請ごとに答えます。</t>
+          <t>オフにすると、リーダーが申請ごとに承認します。</t>
         </is>
       </c>
       <c r="D884" t="inlineStr">
         <is>
-          <t>Off: the leader answers each request.</t>
+          <t>Off: the leader approves each request.</t>
         </is>
       </c>
     </row>
@@ -15780,6 +15780,57 @@
       <c r="D896" t="inlineStr">
         <is>
           <t>{0} items</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_note_title</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>ホストとして使うあなたのルールです。次にホストするゲームに使われます。</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>Your rules as host. They are used the next time you host a game.</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>emp_ui_play_refresh</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>もう一度探す</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>Search again</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>emp_ui_land_go_team</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>チームページを開く</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>Open the Team page</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
World rules: selectable preset cards with a Current chip, compact difference links, custom preset text
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D899"/>
+  <dimension ref="A1:D900"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -15834,6 +15834,23 @@
         </is>
       </c>
     </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_preset_custom</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>自分で選んだルール。下の項目を自由に変更できます。</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>Your own mix: change any rule below by hand.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Play page: official server card first, buttons fit their labels, texts EN/JP/CN
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D900"/>
+  <dimension ref="A1:D902"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3031,12 +3031,12 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>デポから世界を取り出してホストする</t>
+          <t>共有ワールドをホストする</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Take the world from the depot and host it</t>
+          <t>Host the shared world</t>
         </is>
       </c>
     </row>
@@ -15851,6 +15851,40 @@
         </is>
       </c>
     </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>emp_ui_official_title</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>公式サーバー</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>Official server</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>emp_ui_official_open</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>開放中、{0}/{1}人</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>Open, {0}/{1} players</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Official public-server preset, fixed rules, restart warning that stops
SettingsTable: Official preset (index 3), OfficialFixedValues applied at session start and refused by Write while
hosting the official server; rows greyed. Restart warning ends in server.stop on a -empserver game. Bench helper
and preset check.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D899"/>
+  <dimension ref="A1:D901"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -15834,6 +15834,40 @@
         </is>
       </c>
     </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_opt_preset_official</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>公開サーバー（公式）</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>Public server (official)</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_preset_official</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>公開サーバー向け：誰でも参加でき、各自が自分のキャラクターと物語を持ちます。ワールドの持ち出しや非公開化はできず、チームごとに領地を持ちます。</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>For a server open to everyone: each player has their own characters and story, teams hold their own lands, and the world cannot be copied away or hidden.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hub settings as the options window: framed groups, two columns, checkbox first
EmpUi.Box copies LayerConfig's Group (its frame and its small title), Columns
lays two of them side by side. A box setting is the game's checkbox, then its
title and grey line; a choice or a number is its title with the game's
dropdown or slider under it. World rules: each group page is two boxes, the
main rows on the left and the advanced ones on the right (a group without
advanced rows is cut in two), a row kept with the rows under it; the revert is
a small arrow. My settings: boxes, Friends and Ignored side by side; a setting
button is as wide as its label. Lands: a box per land. Not run in game.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D924"/>
+  <dimension ref="A1:D925"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -16259,6 +16259,23 @@
         </is>
       </c>
     </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_adv_title</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>詳細</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hub facts as the character sheet's key/value lines
EmpUi.KeyValue: the game's TopicDefault with its small brown label
right-aligned in its column and the value beside it ('-' when empty). The Play
page's connected state (state, players, host, where) and Help's version use
it. Texts EN/JP/CN (also the labels of the two-page Players and Team views).
Not run in game.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D925"/>
+  <dimension ref="A1:D950"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -16276,6 +16276,431 @@
         </is>
       </c>
     </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_state</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>状態</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_players</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>プレイヤー</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>Players</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_host</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>ホスト</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_where</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>現在地</t>
+        </is>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>Now in</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_version</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>バージョン</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_character</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>キャラクター</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>Character</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_level</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>レベル</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_team</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>チーム</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_ping</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>Ping</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>Ping</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_role</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>役割</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_leader</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>リーダー</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_members</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>メンバー</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>Members</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_joining</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>参加</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>Joining</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_bank</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>チーム銀行</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>Team bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_bills</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>未払いの税</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>Unpaid bills</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_story</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>物語</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>emp_ui_state_connected</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>接続中</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>Connected</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>emp_ui_role_player</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>プレイヤー</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>emp_ui_role_admin</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>管理者</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>emp_ui_role_mod</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>モデレーター</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>Moderator</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>emp_ui_role_frozen</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>凍結中</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>Frozen</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>emp_ui_role_idle</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>離席中</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr">
+        <is>
+          <t>Away from the keyboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>emp_ui_pl_pick</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>左のページでプレイヤーを選んでください。</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>Pick a player on the left page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>emp_ui_pl_actions</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>操作</t>
+        </is>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>Actions</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>emp_ui_team_pick</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>左のページでメンバーを選んでください。</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>Pick a member on the left page.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Play page: buttons where the words start, labels that fit, a guest waiting at the title
Button rows start where the game's note texts start (5 px left of their box);
a fixed-width button is widened to its label at layout time (the label read 0
wide when the button was built and 'Take the world from the depot and host it'
ran out of it). A guest already joined and receiving the world at the title
screen sees where it stands and Disconnect, not the host/join cards (a second
join would drop the first); Disconnect there does not reload the title. The
section headers took the old cards' empty height. Texts EN/JP/CN. Not run in
game.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D950"/>
+  <dimension ref="A1:D951"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -16701,6 +16701,23 @@
         </is>
       </c>
     </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>emp_ui_play_joining</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>ワールドを受け取っています...</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>Receiving the world...</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
TeamOwnGuilds description: on in the Official preset, not off (council 2026-10-28, Q5)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -11254,12 +11254,12 @@
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>「プレイヤーとチームごとの物語」と一緒に：各プレイヤーやチームが戦士、魔術師、盗賊、商人のギルドでも自分の立場を持つ（加入、ランク、貢献、ギルドのクエスト）。チェックした時点の世界のギルドから全員が始める。公式公開サーバーでもオフ。チェックを外す、またはMODなしでセーブを開くと：ホスト自身の物語のギルド。オフ：グループで一つの加入（従来どおり）。</t>
+          <t>「プレイヤーとチームごとの物語」と一緒に：各プレイヤーやチームが戦士、魔術師、盗賊、商人のギルドでも自分の立場を持つ（加入、ランク、貢献、ギルドのクエスト）。チェックした時点の世界のギルドから全員が始める。公式公開サーバーではオン。チェックを外す、またはMODなしでセーブを開くと：ホスト自身の物語のギルド。オフ：グループで一つの加入（従来どおり）。</t>
         </is>
       </c>
       <c r="D632" t="inlineStr">
         <is>
-          <t>With "Each player or team lives its own story": each player or team also has its own place in the Fighters', Mages', Thieves' and Merchants' guilds (membership, rank, contribution, guild quests). Everyone starts with the guilds the world has when the box is ticked. Off on the official public server too. Unticked, or the save opened without the mod: the guilds of the host's own story. Off: one membership for the group, as before.</t>
+          <t>With "Each player or team lives its own story": each player or team also has its own place in the Fighters', Mages', Thieves' and Merchants' guilds (membership, rank, contribution, guild quests). Everyone starts with the guilds the world has when the box is ticked. On on the official public server. Unticked, or the save opened without the mod: the guilds of the host's own story. Off: one membership for the group, as before.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Host box: strangers may visit a player's map (council 2026-10-28, Q4)
MayHost takes visitors of other teams when on (land rules first), 10 visitors per holder with a 'full' line, a stranger holder's upload of a visitor is ignored (only the visitor's own counts), the hourly gold gain cap runs on visitor uploads.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D951"/>
+  <dimension ref="A1:D954"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -16718,6 +16718,57 @@
         </is>
       </c>
     </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>emp_travel_map_full</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>このマップは満員です（訪問者10人まで）</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>This map is full (10 visitors at most).</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_stranger_visits</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>他のチームの人もマップを訪問できる</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>Strangers may visit a player's map</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_stranger_visits</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>ホストの外でマップを持つプレイヤーが、別のチームのプレイヤーも迎え入れます。土地のルールが先に確認され、訪問者は1人のプレイヤーにつき10人までです。訪問者のキャラクター、バッグ、所持金は本人のアップロードだけが有効で、所持金の増加には1時間あたりの上限があります。オフ：公開サーバーでは、チームの仲間、管理者、「許可」された人だけがマップを共有できます。</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>A player holding a map away from the host also takes in players of other teams. Land rules are checked first, and a map takes 10 visitors at most. A visitor's character, bag and gold are taken only from the visitor's own upload (never from the map's holder), and its gold gain has an hourly cap. Off: on a public server only teammates, admins and players let in with "allow" share a map.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Chat flood limit (8 lines / 10 s, 30 s mute notice) and lobby-owner check in OfficialServer.Verify (council 2026-10-28, ops)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D954"/>
+  <dimension ref="A1:D955"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -16769,6 +16769,23 @@
         </is>
       </c>
     </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>emp_chat_flood</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>チャットの書き込みが多すぎます。30秒間ミュートされます。</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>You are typing too fast. Your chat is muted for 30 seconds.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Large crowds box, item 1: players' own steps out of the partial snapshots, full check every 4 s
Host setting LargeCrowds (off by default, on in the Official preset), told to guests as
NetSessionRules key 148. With it on, a player character's entry in a partial
WorldStateSnapshot is kept only when something other than its tile changed (its steps reach
everyone as CharaMoveDelta already), and the full snapshot comes every 20th tick (4 s) instead
of every 5th. The guest's mismatch window grows to 5.2 s so that a character standing still
is still put right by two full snapshots in a row.

Not tested in game (worker without the bench): see bench/crowds_check.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D951"/>
+  <dimension ref="A1:D953"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -16718,6 +16718,40 @@
         </is>
       </c>
     </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_large_crowds</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>大人数：各プレイヤーには近くのものだけを送る</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>Large crowds: send each player only what is near it</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_large_crowds</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>各プレイヤーには、自分のキャラクターの近く（24マス）、仲間、チーム、取引・決闘・戦闘の相手だけを毎回送ります。マップの残りは毎秒1回、マップ全体の確認は4秒ごと。何も消えませんが、遠くのキャラクターはとびとびに動きます。オフ：全員にマップ全体を毎回送ります（従来どおり）。</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>Each player is sent at full rate only what is near its character (24 tiles), its companions, its team and whoever it trades, duels or fights with; the rest of the map once a second, and the whole map is checked every 4 seconds. Nothing disappears; far characters move in steps. Off: every player gets the whole map at full rate, as before.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Host setting "Fast joins and saves for big worlds" and join/save timing logs
Stage 2 of PLAN_100_players, part (a): the join copy (world JSON+LZ4, map save, map
files LZ4, per-peer MessagePack of the world, fragment split) and the dedicated
server's 5-minute save all ran in one frame of the main thread. These logs measure
it: "Join prepared in X ms main thread, Y ms worker" and "Server: save made in X ms
main thread". The setting is off by default and on in the Official preset; it does
nothing yet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D951"/>
+  <dimension ref="A1:D953"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -16718,6 +16718,40 @@
         </is>
       </c>
     </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_fast_joins</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>大きな世界の参加と保存を速く</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>Fast joins and saves for big worlds</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_fast_joins</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>大きな世界向け：プレイヤーの参加と定期保存でゲームが止まる時間を短くします。世界とマップの写しはゲームの中で作り、その圧縮と送信、保存ファイルの書き込みは横で行います。オフ：すべてゲームの中で行います。</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>For big worlds: a player joining and the periodic save freeze the game for everyone for less time. The copy of the world and of the map is still made in the game; compressing and sending it, and writing the save files, are done beside it. Off: all of it is done in the game.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lobby: tell a guest kicked by the host's friend/invited filter (D4)
New text emp_lobby_not_allowed (EN, JP, CN).

Compile-checked only (not run in game).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D959"/>
+  <dimension ref="A1:D960"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -16854,6 +16853,23 @@
         </is>
       </c>
     </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>emp_lobby_not_allowed</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>このゲームはホストの Steam フレンドか招待されたプレイヤーのみ参加できます。</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>This game only accepts the host's Steam friends or invited players.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
World rules tab: equal-height framed preset cards, 4 sub-tab pills, full differences list with values
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D963"/>
+  <dimension ref="A1:D964"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -16922,6 +16921,23 @@
         </is>
       </c>
     </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_diff_line</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>{0}：{1}（おすすめ：{2}）</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>{0}: {1} (recommended: {2})</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Polish Team, Lands and Server info pages: scrolling team list, character-sheet member facts, illustrated empty states
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D963"/>
+  <dimension ref="A1:D965"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11424,12 +11424,14 @@
       </c>
       <c r="C642" t="inlineStr">
         <is>
-          <t>ホストはまだ何も書いていません。</t>
+          <t>ホストはまだ何も書いていません。
+書かれるとここに表示されます。</t>
         </is>
       </c>
       <c r="D642" t="inlineStr">
         <is>
-          <t>The host hasn't written anything yet.</t>
+          <t>The host hasn't written anything yet.
+It will show up here once they do.</t>
         </is>
       </c>
     </row>
@@ -12138,12 +12140,14 @@
       </c>
       <c r="C684" t="inlineStr">
         <is>
-          <t>あなたはチームに入っていません（放浪者です）。</t>
+          <t>あなたはチームに入っていません（放浪者です）。
+チームを作るか、他のチームに参加しましょう。</t>
         </is>
       </c>
       <c r="D684" t="inlineStr">
         <is>
-          <t>You are not in a team (you are a Wanderer).</t>
+          <t>You are not in a team (you are a Wanderer).
+Found a team, or join one from the list.</t>
         </is>
       </c>
     </row>
@@ -14363,12 +14367,14 @@
       </c>
       <c r="C813" t="inlineStr">
         <is>
-          <t>まだ何も書いていません。参加者全員に表示されます。</t>
+          <t>まだ何も書いていません。
+書いた内容は参加者全員に表示されます。</t>
         </is>
       </c>
       <c r="D813" t="inlineStr">
         <is>
-          <t>Nothing written yet. Every player can read it here.</t>
+          <t>Nothing written yet.
+What you write is shown to every player.</t>
         </is>
       </c>
     </row>
@@ -15400,12 +15406,14 @@
       </c>
       <c r="C874" t="inlineStr">
         <is>
-          <t>このワールドではチームは無効です。</t>
+          <t>このワールドではチームが無効です。
+チームを使うには、ホストがワールドのルールでオンにします。</t>
         </is>
       </c>
       <c r="D874" t="inlineStr">
         <is>
-          <t>Teams are off in this world.</t>
+          <t>Teams are off in this world.
+The host can turn them on in the World rules.</t>
         </is>
       </c>
     </row>
@@ -15417,12 +15425,14 @@
       </c>
       <c r="C875" t="inlineStr">
         <is>
-          <t>このワールドではチームは無効です。ホストだけがオンにできます。</t>
+          <t>このワールドではチームが無効です。
+オンにできるのはホストだけです。</t>
         </is>
       </c>
       <c r="D875" t="inlineStr">
         <is>
-          <t>Teams are off in this world. Only the host can turn them on.</t>
+          <t>Teams are off in this world.
+Only the host can turn them on.</t>
         </is>
       </c>
     </row>
@@ -15451,12 +15461,12 @@
       </c>
       <c r="C877" t="inlineStr">
         <is>
-          <t>オンにする</t>
+          <t>ワールドのルールでチームをオンにする</t>
         </is>
       </c>
       <c r="D877" t="inlineStr">
         <is>
-          <t>Turn on</t>
+          <t>Turn on teams in World rules</t>
         </is>
       </c>
     </row>
@@ -15638,12 +15648,14 @@
       </c>
       <c r="C888" t="inlineStr">
         <is>
-          <t>まだ土地がありません。野原で土地の権利書を読むと手に入ります。</t>
+          <t>まだ土地がありません。
+野原で土地の権利書を読むと手に入ります。</t>
         </is>
       </c>
       <c r="D888" t="inlineStr">
         <is>
-          <t>No land yet. Read a land deed on a field to claim one.</t>
+          <t>No land yet.
+Read a land deed on a field to claim one.</t>
         </is>
       </c>
     </row>
@@ -15655,12 +15667,14 @@
       </c>
       <c r="C889" t="inlineStr">
         <is>
-          <t>土地を持つには、まずチームを作るか参加してください。</t>
+          <t>土地を持つには、チームが必要です。
+まずチームを作るか参加してください。</t>
         </is>
       </c>
       <c r="D889" t="inlineStr">
         <is>
-          <t>Found or join a team to hold land.</t>
+          <t>Land belongs to a team.
+Found or join a team to hold some.</t>
         </is>
       </c>
     </row>
@@ -16919,6 +16933,40 @@
       <c r="D963" t="inlineStr">
         <is>
           <t>The game's mods were not loaded: {0} contains code (DLL). Tick "Also code mods (DLL)" in Client settings only if you trust this host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>emp_ui_team_leader_short</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>{0}　·　メンバー{1}人</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>{0}  ·  {1} members</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>emp_ui_team_join_short</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>参加</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>Join</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Polish the multiplayer menu: player search/sort/team filter and paging, detail facts, rules rows, one settings page, help links, fitted tab strip, debug box hidden while open
Compile-checked only, not run in game.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D963"/>
+  <dimension ref="A1:D975"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -16922,6 +16922,210 @@
         </is>
       </c>
     </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>emp_ui_pl_search</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>名前で検索</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>Search by name</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>emp_ui_pl_sort</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>並び順：{0}</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>Sort: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>emp_ui_pl_sort_name</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>名前</t>
+        </is>
+      </c>
+      <c r="D966" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>emp_ui_pl_sort_level</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>レベル</t>
+        </is>
+      </c>
+      <c r="D967" t="inlineStr">
+        <is>
+          <t>level</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>emp_ui_pl_sort_ping</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>遅延</t>
+        </is>
+      </c>
+      <c r="D968" t="inlineStr">
+        <is>
+          <t>ping</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>emp_ui_pl_sort_team</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>チーム</t>
+        </is>
+      </c>
+      <c r="D969" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>emp_ui_pl_myteam</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>自分のチーム</t>
+        </is>
+      </c>
+      <c r="D970" t="inlineStr">
+        <is>
+          <t>My team</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>emp_ui_pl_none</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>該当するプレイヤーはいません。</t>
+        </is>
+      </c>
+      <c r="D971" t="inlineStr">
+        <is>
+          <t>No player matches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>emp_ui_pl_page</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>{0} / {1}</t>
+        </is>
+      </c>
+      <c r="D972" t="inlineStr">
+        <is>
+          <t>{0} / {1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>emp_ui_rules_summary</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>適用中のルール {0} 件、先頭の数件を表示。</t>
+        </is>
+      </c>
+      <c r="D973" t="inlineStr">
+        <is>
+          <t>{0} rules in force, the first ones here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>emp_ui_rules_open</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>ルールを編集</t>
+        </is>
+      </c>
+      <c r="D974" t="inlineStr">
+        <is>
+          <t>Edit the rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>emp_ui_help_open</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>開く：{0}</t>
+        </is>
+      </c>
+      <c r="D975" t="inlineStr">
+        <is>
+          <t>Open: {0}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hub features WP0: four host boxes, rules keys 149-152, stub deltas 1230-1232, Journal and Leaderboards tabs
Compile-checked only.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D978"/>
+  <dimension ref="A1:D996"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -17191,6 +17191,312 @@
         </is>
       </c>
     </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_team_sheets</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>チームメイトのキャラクターシート</t>
+        </is>
+      </c>
+      <c r="D979" t="inlineStr">
+        <is>
+          <t>Teammates' character sheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_team_sheets</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>チームメイトの読み取り専用キャラクターシートを、ホストから受け取って開けます。オフ：シートはありません。</t>
+        </is>
+      </c>
+      <c r="D980" t="inlineStr">
+        <is>
+          <t>Players can open a read-only character sheet of their teammates, sent by the host. Off: no sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_activity_journal</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>活動の記録</t>
+        </is>
+      </c>
+      <c r="D981" t="inlineStr">
+        <is>
+          <t>Activity journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_activity_journal</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>ホストが世界の出来事（チーム結成、決闘の勝利、ボス討伐、死亡、記録）を記録し、「記録」ページに表示します。オフ：記録はありません。</t>
+        </is>
+      </c>
+      <c r="D982" t="inlineStr">
+        <is>
+          <t>The host keeps a journal of the world's events (teams founded, duels won, boss kills, deaths, records), shown on the Journal page. Off: no journal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_team_banner</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>チームの旗</t>
+        </is>
+      </c>
+      <c r="D983" t="inlineStr">
+        <is>
+          <t>Team banners</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_team_banner</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>各チームのリーダーが紋章と色を選び、チームのページに表示します。オフ：旗はありません。</t>
+        </is>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>Each team gets a banner (an emblem and a colour) chosen by its leader and shown on the Teams page. Off: no banners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_cfg_leaderboards</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>ランキング</t>
+        </is>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>Leaderboards</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>emp_ui_sv_desc_leaderboards</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>ホストがプレイヤーとチームを順位付け（レベル、最深階、決闘の勝利、チームの資産）し、「ランキング」ページに表示します。オフ：順位はありません。</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>The host ranks players and teams (level, deepest floor, duels won, team wealth), shown on the Leaderboards page. Off: no rankings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>emp_ui_tab_journal</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>emp_tab_journal</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>記録</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>Journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_journal</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>世界の出来事の記録</t>
+        </is>
+      </c>
+      <c r="D989" t="inlineStr">
+        <is>
+          <t>What happened in the world</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>emp_ui_tab_leaderboard</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>ランキング</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>Leaderboards</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>emp_tab_leaderboard</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>ランキング</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>Leaderboards</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_leaderboard</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>プレイヤーとチームの順位</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>Rankings of players and teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>emp_ui_journal_off</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>このワールドでは活動の記録はオフです。</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>The activity journal is off in this world.</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>emp_ui_journal_empty</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>まだ記録はありません。</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>Nothing in the journal yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>emp_ui_leaderboard_off</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>このワールドではランキングはオフです。</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>Leaderboards are off in this world.</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>emp_ui_leaderboard_empty</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>まだ順位はありません。</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>No rankings yet.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leaderboards: host-authoritative boards (level, deepest floor, duels won, team wealth), tab, texts
Compile-checked only, not run in game. dev/_tools/leaderboard_check.py written, not run.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D996"/>
+  <dimension ref="A1:D1003"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -17497,6 +17496,125 @@
         </is>
       </c>
     </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>emp_ui_lb_level</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>レベル</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>emp_ui_lb_deepest</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>最深階</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>Deepest floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>emp_ui_lb_duels</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>決闘の勝利</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>Duels won</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>emp_ui_lb_wealth</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>チームの資産</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>Team wealth</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>emp_ui_lb_you</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>あなた</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>emp_ui_lb_rank</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>{0}位（{1}）</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>Rank {0} ({1})</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>emp_ui_lb_unranked</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>順位なし</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>Not ranked</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Team character sheets (package A): Sheet button, host-checked CharaSheetDelta, read-only LayerChara on a throwaway chara
Compile-checked only, not run in game.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D996"/>
+  <dimension ref="A1:D997"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -17497,6 +17497,23 @@
         </is>
       </c>
     </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>emp_ui_team_sheet</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>キャラシート</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Activity journal (hub plan B): host ring of 200 events saved in the world, JournalDelta, Journal tab with filters
Harmony postfixes on team found/join/leave, land claimed/lost, duel won, player death, boss kill, record depth. Team-only entries go to that team's peers only. Compile-checked only; dev/_tools/journal_check.py not run.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D996"/>
+  <dimension ref="A1:D1009"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -17497,6 +17496,227 @@
         </is>
       </c>
     </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>emp_journal_1</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>{0}がチーム「{1}」を結成した。</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>{0} founded the team {1}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>emp_journal_2</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>{0}がチーム「{1}」に加わった。</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>{0} joined the team {1}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>emp_journal_3</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>{0}がチーム「{1}」を抜けた。</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>{0} left the team {1}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>emp_journal_4</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>{0}が{1}のために土地「{2}」を確保した。</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>{0} claimed the land {2} for {1}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>emp_journal_5</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>{1}は不在のため土地{2}か所を失った。</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>{1} lost {2} land(s) after being away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>emp_journal_6</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>{0}が{2}との決闘に勝った。</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>{0} won a duel against {2}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>emp_journal_7</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>{0}が{2}で死んだ。</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>{0} died in {2}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>emp_journal_8</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>{0}が{2}を倒した。</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>{0} defeated {2}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>emp_journal_9</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>{0}が最深記録を更新した：危険度{2}。</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>{0} reached a new record depth: danger {2}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>emp_ui_journal_filter</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>表示</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>Show</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>emp_ui_journal_f_all</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>すべて</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>emp_ui_journal_f_team</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>チーム</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>emp_ui_journal_f_mine</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>自分</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>Mine</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Team banners (package C): emblem and colour chosen by the leader, host-kept, shown on the Team page, land map, journal hook
Compile-checked only; not run in game.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1004"/>
+  <dimension ref="A1:D1013"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -17633,6 +17632,159 @@
         </is>
       </c>
     </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>emp_ui_team_banner</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>チームの旗</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>Banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>emp_ui_team_banner_tool</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>旗を選ぶ</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>Banner</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>emp_ui_team_banner_emblem</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>紋章</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>Emblem</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>emp_ui_team_banner_color</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>色</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>Colour</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>emp_ui_team_lands_map</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>土地の地図</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>Land map</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>emp_ui_team_lands_none</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>土地はまだありません</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>No land yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>emp_ui_team_lands_hover</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>点にカーソルを合わせると土地名が出ます</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>Hover a dot for the land name</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>emp_ui_team_journal</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>チームの記録</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>Team journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>emp_ui_team_journal_none</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>まだ何もありません</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>Nothing yet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Team banner: the leader picks any item of the game as the emblem
New TeamsDelta Key(10) Things and host storage team_things (old Key 9 and team_banners still read); the request carries the source id, the host refuses unknown ids; picker with search and 30-per-page icons; EN/JP/CN texts. Compile-checked only.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1026"/>
+  <dimension ref="A1:D1027"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -18007,6 +18007,24 @@
         </is>
       </c>
     </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>emp_ui_team_banner_search</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr"/>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>名前かIDで検索</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>Search any item by name or id</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hub polish: tab strip fits, one-line player rows with team chip and styled search, bigger team logo, fixed leaderboard rows and clearer own rank (compile-checked only)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -16995,12 +16995,12 @@
       </c>
       <c r="C967" t="inlineStr">
         <is>
-          <t>名前で検索</t>
+          <t>プレイヤーを検索</t>
         </is>
       </c>
       <c r="D967" t="inlineStr">
         <is>
-          <t>Search by name</t>
+          <t>Search a player</t>
         </is>
       </c>
     </row>
@@ -17590,12 +17590,12 @@
       </c>
       <c r="C1002" t="inlineStr">
         <is>
-          <t>あなた</t>
+          <t>あなたの順位</t>
         </is>
       </c>
       <c r="D1002" t="inlineStr">
         <is>
-          <t>You</t>
+          <t>Your rank</t>
         </is>
       </c>
     </row>
@@ -17607,12 +17607,12 @@
       </c>
       <c r="C1003" t="inlineStr">
         <is>
-          <t>{0}位（{1}）</t>
+          <t>{1}人中{0}位（{2}）</t>
         </is>
       </c>
       <c r="D1003" t="inlineStr">
         <is>
-          <t>Rank {0} ({1})</t>
+          <t>{0} of {1} ({2})</t>
         </is>
       </c>
     </row>
@@ -18013,7 +18013,6 @@
           <t>emp_ui_team_banner_search</t>
         </is>
       </c>
-      <c r="B1027" t="inlineStr"/>
       <c r="C1027" t="inlineStr">
         <is>
           <t>名前かIDで検索</t>

</xml_diff>

<commit_message>
Tabs keep the game's font: no label shrinking, Journal and Leaderboards merged into a Community tab, Help moved into Server info; team logo can be a monster (typed t:/c: ids, Items/Monsters pills). Compile-checked only
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1027"/>
+  <dimension ref="A1:D1033"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -18020,7 +18020,109 @@
       </c>
       <c r="D1027" t="inlineStr">
         <is>
-          <t>Search any item by name or id</t>
+          <t>Search by name or id</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>emp_ui_tab_community</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>コミュニティ</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>emp_tab_community</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>コミュニティ</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_community</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>世界の記録とランキング</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>The world journal and the leaderboards</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>emp_ui_lb_board</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>ランキング</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>Board</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>emp_ui_team_banner_items</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>アイテム</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>emp_ui_team_banner_monsters</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>モンスター</t>
+        </is>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>Monsters</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Team emblem editor in the Team page banner card
The leader builds the emblem from up to 8 sprites: a 3x preview of the baked draft, the layer list (select, up,
down, remove), Add layer through the Items/Monsters picker (now given an onPick callback), nudges of 2, size -/+
and a slider, rotate 90, flip H/V, tint swatches and none, background colour and shape pills (square, round,
shield), Undo (20 steps), Reset and Save, which asks the host with the canonical text. The draft stays local
until Save. Texts in EN, JP and CN. Compile-checked only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1033"/>
+  <dimension ref="A1:D1051"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -18126,6 +18126,312 @@
         </is>
       </c>
     </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_layers</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>レイヤー（{0}/{1}）</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>Layers ({0}/{1})</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_add</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>レイヤーを追加</t>
+        </is>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>Add layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_add_close</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>一覧を閉じる</t>
+        </is>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>Close the list</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_selected</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>選択中のレイヤー：{0}</t>
+        </is>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>Selected layer: {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_move</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>移動</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>Move</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_size</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>大きさ</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_rotate</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>90°回転</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>Rotate 90°</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_flip_h</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>左右反転</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>Flip horizontally</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_flip_v</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>上下反転</t>
+        </is>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>Flip vertically</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_tint</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>色合い</t>
+        </is>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>Tint</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_tint_none</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>なし</t>
+        </is>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_background</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>背景</t>
+        </is>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>Background</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_square</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>四角</t>
+        </is>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>Square</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_round</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>丸</t>
+        </is>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_shield</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>盾</t>
+        </is>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>Shield</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_undo</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>元に戻す</t>
+        </is>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>Undo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_reset</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>リセット</t>
+        </is>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>Reset</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_save</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>保存</t>
+        </is>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>Save</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Team tab: Team and Emblem sub-tabs, other teams list fixed
The emblem editor sat below the visible area of the Team page. It now has its own Emblem sub-tab laid out as two
pages (preview, background, shape and buttons on the left; layers, tools or picker on the right); non-leaders see a
read-only view. Other teams no longer lists the player's own team or empty ghost teams, and names the first member
when the book has no leader. Compile-checked only, not run in game.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1051"/>
+  <dimension ref="A1:D1053"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -18432,6 +18431,40 @@
         </is>
       </c>
     </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>emp_ui_team_tab_team</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>チーム</t>
+        </is>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>emp_ui_team_tab_emblem</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>エンブレム</t>
+        </is>
+      </c>
+      <c r="D1053" t="inlineStr">
+        <is>
+          <t>Emblem</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hub: Chat tab with history and a team channel; clearer characters list, rank line and empty emblem page
- ChatLog keeps the lines this game was shown (everyone, team, private, server; 200 at most, memory only). The Chat tab
  filters them, adds new ones live without being rebuilt (a typed line keeps its text), and sends to everyone, the
  team (MsgSayDelta.Team: the host checks the speaker's team and relays to that team's members only) or one player.
- Players > Characters: portraits, and the character alone when the Steam name is unknown (not a raw id).
- Leaderboards: "#1 of 3 players, score 1"; the empty emblem layer list says how to start.
Tested: leaderboard_check 9/9, team_emblem_check 23/23, screenshots. The Chat tab is compile-checked only
(chat_tab_check.py written, run pending).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1095"/>
+  <dimension ref="A1:D1112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -17607,12 +17607,12 @@
       </c>
       <c r="C1003" t="inlineStr">
         <is>
-          <t>{1}人中{0}位（{2}）</t>
+          <t>{1}人中{0}位、スコア {2}</t>
         </is>
       </c>
       <c r="D1003" t="inlineStr">
         <is>
-          <t>{0} of {1} ({2})</t>
+          <t>#{0} of {1} players, score {2}</t>
         </is>
       </c>
     </row>
@@ -19177,6 +19177,295 @@
       <c r="D1095" t="inlineStr">
         <is>
           <t>Starters</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>emp_ui_saved_chars_line_alone</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>{0}（Lv {1}）</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>{0} (Lv {1})</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_start</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>まだレイヤーがありません。「レイヤーを追加」でゲームのアイテムやモンスターを選ぶか、左の「ひな形」から始めましょう。</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>No layer yet. Press Add layer to pick any item or monster of the game, or start from Starters on the left.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>emp_ui_tab_chat</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>チャット</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_chat</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>みんな、チーム、個人宛てのメッセージ</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>Messages: everyone, your team, private</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_off</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>マルチプレイ中にチャットできます。</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>Chat works in a multiplayer game.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_show</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>表示</t>
+        </is>
+      </c>
+      <c r="D1101" t="inlineStr">
+        <is>
+          <t>Show</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_all</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>すべて</t>
+        </is>
+      </c>
+      <c r="D1102" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_everyone</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>全員</t>
+        </is>
+      </c>
+      <c r="D1103" t="inlineStr">
+        <is>
+          <t>Everyone</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_map</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>このマップ</t>
+        </is>
+      </c>
+      <c r="D1104" t="inlineStr">
+        <is>
+          <t>This map</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_team</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>チーム</t>
+        </is>
+      </c>
+      <c r="D1105" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_private</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>個人</t>
+        </is>
+      </c>
+      <c r="D1106" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_server</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>サーバー</t>
+        </is>
+      </c>
+      <c r="D1107" t="inlineStr">
+        <is>
+          <t>Server</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_to</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>{0} へ</t>
+        </is>
+      </c>
+      <c r="D1108" t="inlineStr">
+        <is>
+          <t>To {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_hint</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>メッセージを入力…</t>
+        </is>
+      </c>
+      <c r="D1109" t="inlineStr">
+        <is>
+          <t>Write a message…</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_send</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>送信</t>
+        </is>
+      </c>
+      <c r="D1110" t="inlineStr">
+        <is>
+          <t>Send</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_empty</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>まだメッセージはありません。</t>
+        </is>
+      </c>
+      <c r="D1111" t="inlineStr">
+        <is>
+          <t>No message yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>emp_ui_chat_team_tag</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>{0}（チーム）</t>
+        </is>
+      </c>
+      <c r="D1112" t="inlineStr">
+        <is>
+          <t>{0} (team)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Richer player card in the Players tab: title, race/job, team emblem, time here, records, recent deeds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1112"/>
+  <dimension ref="A1:D1120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -19469,6 +19468,142 @@
         </is>
       </c>
     </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_title</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>称号</t>
+        </is>
+      </c>
+      <c r="D1113" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_race_job</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>種族・職業</t>
+        </is>
+      </c>
+      <c r="D1114" t="inlineStr">
+        <is>
+          <t>Race, job</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_session</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>今回の滞在</t>
+        </is>
+      </c>
+      <c r="D1115" t="inlineStr">
+        <is>
+          <t>Here for</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_deepest</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>最深階</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr">
+        <is>
+          <t>Deepest floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>emp_ui_kv_duels</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>決闘の勝利</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>Duels won</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>emp_ui_pl_deeds</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>最近の行い</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>Recent deeds</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>emp_ui_time_hm</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>{0}時間{1}分</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>{0} h {1} min</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>emp_ui_time_m</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>{0}分</t>
+        </is>
+      </c>
+      <c r="D1120" t="inlineStr">
+        <is>
+          <t>{0} min</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hub: Server info > Status page (host, players, teams, world date, session time, ping, restart, versions)
Compile-checked.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1120"/>
+  <dimension ref="A1:D1131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -467,6 +467,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -19604,6 +19605,193 @@
         </is>
       </c>
     </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>emp_info_status</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>サーバーの状態</t>
+        </is>
+      </c>
+      <c r="D1121" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>emp_info_status_off</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>マルチプレイ中に表示されます。</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>Shown in a multiplayer game.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>emp_info_st_host</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>ホスト</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>Host</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>emp_info_st_players</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>オンラインのプレイヤー</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>Players online</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>emp_info_st_teams</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>チーム</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>Teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>emp_info_st_date</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>世界の日付</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>World date</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>emp_info_st_session</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>このセッション</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>This session</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>emp_info_st_ping</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>ping</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>Ping</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>emp_info_st_restart</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>再起動まで</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>Restart in</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>emp_info_st_mod</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>Elin Together</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>Elin Together</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>emp_info_st_game</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Elin</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>Elin</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Emblem editor: small previews at list sizes, Mirror (symmetric copy of a layer), Save lit only with unsaved changes
Tested: team_emblem_check 23/23, screenshots of the editor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1233"/>
+  <dimension ref="A1:D1235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -21526,6 +21526,40 @@
         </is>
       </c>
     </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_mirror</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>左右対称</t>
+        </is>
+      </c>
+      <c r="D1234" t="inlineStr">
+        <is>
+          <t>Mirror</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>emp_ui_emblem_unsaved</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>未保存の変更があります。</t>
+        </is>
+      </c>
+      <c r="D1235" t="inlineStr">
+        <is>
+          <t>Unsaved changes.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Say "Elin Together public server", never "official": it is the mod team's server, not the game developer's (user 2026-10-30)
Player texts (EN, JP, CN), the welcome message and the setting descriptions.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -9455,12 +9455,12 @@
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>★ Elin Together 公式サーバー</t>
+          <t>★ Elin Together 公開サーバー</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
         <is>
-          <t>★ Official Elin Together server</t>
+          <t>★ Elin Together public server</t>
         </is>
       </c>
     </row>
@@ -9472,12 +9472,12 @@
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>公式サーバーに参加</t>
+          <t>Elin Together 公開サーバーに参加</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
         <is>
-          <t>Join the official server</t>
+          <t>Join the Elin Together public server</t>
         </is>
       </c>
     </row>
@@ -9795,12 +9795,12 @@
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>公式サーバーは今は開いていません</t>
+          <t>Elin Together 公開サーバーは今は開いていません</t>
         </is>
       </c>
       <c r="D547" t="inlineStr">
         <is>
-          <t>The official server is not open right now</t>
+          <t>The Elin Together public server is not open right now</t>
         </is>
       </c>
     </row>
@@ -9812,12 +9812,12 @@
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>公式サーバーではキャラクターの持ち込みはできません</t>
+          <t>Elin Together 公開サーバーではキャラクターの持ち込みはできません</t>
         </is>
       </c>
       <c r="D548" t="inlineStr">
         <is>
-          <t>The official server does not take imported characters</t>
+          <t>The Elin Together public server does not take imported characters</t>
         </is>
       </c>
     </row>
@@ -10991,12 +10991,12 @@
       </c>
       <c r="C617" t="inlineStr">
         <is>
-          <t>公式サーバーでは常にオン：プレイヤーとチームごと。</t>
+          <t>Elin Together 公開サーバーでは常にオン：プレイヤーとチームごと。</t>
         </is>
       </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>Always on for the official public server: one for each player and team.</t>
+          <t>Always on for the Elin Together public server: one for each player and team.</t>
         </is>
       </c>
     </row>
@@ -11254,12 +11254,12 @@
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>「プレイヤーとチームごとの物語」と一緒に：各プレイヤーやチームが戦士、魔術師、盗賊、商人のギルドでも自分の立場を持つ（加入、ランク、貢献、ギルドのクエスト）。チェックした時点の世界のギルドから全員が始める。公式公開サーバーではオン。チェックを外す、またはMODなしでセーブを開くと：ホスト自身の物語のギルド。オフ：グループで一つの加入（従来どおり）。</t>
+          <t>「プレイヤーとチームごとの物語」と一緒に：各プレイヤーやチームが戦士、魔術師、盗賊、商人のギルドでも自分の立場を持つ（加入、ランク、貢献、ギルドのクエスト）。チェックした時点の世界のギルドから全員が始める。Elin Together 公開サーバーではオン。チェックを外す、またはMODなしでセーブを開くと：ホスト自身の物語のギルド。オフ：グループで一つの加入（従来どおり）。</t>
         </is>
       </c>
       <c r="D632" t="inlineStr">
         <is>
-          <t>With "Each player or team lives its own story": each player or team also has its own place in the Fighters', Mages', Thieves' and Merchants' guilds (membership, rank, contribution, guild quests). Everyone starts with the guilds the world has when the box is ticked. On on the official public server. Unticked, or the save opened without the mod: the guilds of the host's own story. Off: one membership for the group, as before.</t>
+          <t>With "Each player or team lives its own story": each player or team also has its own place in the Fighters', Mages', Thieves' and Merchants' guilds (membership, rank, contribution, guild quests). Everyone starts with the guilds the world has when the box is ticked. On on the Elin Together public server. Unticked, or the save opened without the mod: the guilds of the host's own story. Off: one membership for the group, as before.</t>
         </is>
       </c>
     </row>
@@ -14248,12 +14248,12 @@
       </c>
       <c r="C806" t="inlineStr">
         <is>
-          <t>公式サーバーでは使えません</t>
+          <t>Elin Together 公開サーバーでは使えません</t>
         </is>
       </c>
       <c r="D806" t="inlineStr">
         <is>
-          <t>Not available on the official server</t>
+          <t>Not available on the Elin Together public server</t>
         </is>
       </c>
     </row>
@@ -15873,12 +15873,12 @@
       </c>
       <c r="C901" t="inlineStr">
         <is>
-          <t>公式サーバー</t>
+          <t>Elin Together 公開サーバー</t>
         </is>
       </c>
       <c r="D901" t="inlineStr">
         <is>
-          <t>Official server</t>
+          <t>Elin Together public server</t>
         </is>
       </c>
     </row>
@@ -15907,12 +15907,12 @@
       </c>
       <c r="C903" t="inlineStr">
         <is>
-          <t>公開サーバー（公式）</t>
+          <t>Elin Together 公開サーバー</t>
         </is>
       </c>
       <c r="D903" t="inlineStr">
         <is>
-          <t>Public server (official)</t>
+          <t>Elin Together public server</t>
         </is>
       </c>
     </row>
@@ -16230,12 +16230,12 @@
       </c>
       <c r="C922" t="inlineStr">
         <is>
-          <t>公式サーバーが設定</t>
+          <t>Elin Together 公開サーバーが設定</t>
         </is>
       </c>
       <c r="D922" t="inlineStr">
         <is>
-          <t>Set by the official server</t>
+          <t>Set by the Elin Together public server</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Report a bug: a tab of its own, the form laid out like the game's Report Bugs window
Category, one-line summary, detail box, does it happen again, video/picture/logs boxes, tips on the right page; the
game picture is taken before the window opened. Tested: bug_report_check 35/35, replay_pause_check 4/4, screenshot.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1266"/>
+  <dimension ref="A1:D1267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -22087,6 +22087,23 @@
         </is>
       </c>
     </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>emp_tip_tab_report</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>不具合を開発者に報告</t>
+        </is>
+      </c>
+      <c r="D1267" t="inlineStr">
+        <is>
+          <t>Tell the developers about a bug</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>